<commit_message>
Bilingual public site (RU/EN) and real tariff pricing
i18n:
- Cookie-based locale (RU default) with a RU|EN switcher in the header;
  dictionaries cover the landing, payment, support and login pages, the
  nav/footer, and the AI widget (greeting, chat labels, suggestions).
- The client assistant receives an interface-language hint and defaults
  to English for EN visitors; voice dictation follows the site language.
- Client cabinet and admin workspace remain Russian for now.

Pricing (set by the founder):
- 5 weeks: $1,200 + 5% service fee + $180 formula delivery = $1,440
  (Karen sends his formula as a gift with the plan).
- 100 days: $3,500 + 5% service fee = $3,675.
- Payment page shows price breakdowns; product label renamed to
  «100 дней»; assistant prompts updated with exact tariffs.
- Financial model updated with the real prices (verified to the dollar)
  plus a gift-cost input; 414 formulas recalculated error-free.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/launch/Финансовая_модель_Python_Method.xlsx
+++ b/docs/launch/Финансовая_модель_Python_Method.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="128">
   <si>
     <t xml:space="preserve">Финансовая модель Python Method Center — «Реабилитация без границ»</t>
   </si>
@@ -50,7 +50,10 @@
     <t xml:space="preserve">• Стоимость инфраструктуры и ИИ — фактические тарифы Vercel/Supabase/Anthropic/OpenAI, июль 2026.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Цены тарифов, оценка среднего чека и зарплаты помечены как ПРЕДПОЛОЖЕНИЯ — замените реальными значениями.</t>
+    <t xml:space="preserve">• Цены — факт от 23.07.2026: «5 недель» $1200 (+5% сбор, +$180 доставка формулы-подарка) = $1440; «100 дней» $3500 (+5% сбор) = $3675.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Жёлтым остались: доля «100 дней», продления, рост, себестоимость подарка, зарплаты, маркетинг, раунд — заполните.</t>
   </si>
   <si>
     <t xml:space="preserve">Листы:</t>
@@ -92,258 +95,279 @@
     <t xml:space="preserve">Цена тарифа «5 недель», $</t>
   </si>
   <si>
-    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — замените реальной ценой.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Цена тарифа «15 недель», $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Доля клиентов, выбирающих «15 недель»</t>
+    <t xml:space="preserve">ФАКТ — установлено основателем 23.07.2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цена тарифа «100 дней», $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сервисный сбор, % к каждому тарифу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ФАКТ — 5% добавляется к сумме тарифа.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доставка формулы (тариф «5 недель»), $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ФАКТ — формула отправляется Кареном в подарок, клиент оплачивает доставку $180.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Себестоимость формулы и доставки, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — во сколько центру обходится формула + отправка. Замените фактом.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля клиентов, выбирающих «100 дней»</t>
   </si>
   <si>
     <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — оцените по вашим 480 кейсам.</t>
   </si>
   <si>
+    <t xml:space="preserve">Средний чек (с сбором и доставкой), $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 недель: $1200×1,05+$180=$1440; 100 дней: $3500×1,05=$3675. Средневзвешенно. Формула.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля клиентов, продлевающих сопровождение</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — доля повторных покупок после завершения тарифа.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">РОСТ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рост новых клиентов, % в месяц (базовый сценарий)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Базовый: +8% в месяц. Сценарии — на листе «Сценарии».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ЗАТРАТЫ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Эквайринг Stripe, % от выручки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,9% + $0,30 за транзакцию ≈ 3,2% при среднем чеке. Тариф Stripe US, июль 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ИИ-затраты на активного клиента в месяц, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Оценка из фактических тарифов Claude/GPT при текущем режиме «Лучший ответ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Инфраструктура (Vercel, Supabase Pro, домен), $/мес</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Факт: Supabase Pro $25 + Vercel Pro ~$20 + резерв. Фиксированные.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Команда (Карен, Анна, поддержка), $/мес — год 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — суммарные выплаты команде. Замените реальными.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рост затрат на команду в год 2 (множитель)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ: расширение команды на 2-м году.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маркетинг, % от выручки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — бюджет привлечения.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Юристы, бухгалтерия, прочее, $/мес</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ИНВЕСТИЦИИ И ПРИВЛЕЧЕНИЕ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Запрашиваемый раунд, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — сумма, которую вы просите у инвестора.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стоимость привлечения клиента (CAC), $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ = маркетинг на клиента. Проверится фактом первых месяцев.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Помесячный прогноз (базовый сценарий)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Показатель</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">М24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Новые клиенты</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Продажи «5 недель», шт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Продажи «100 дней», шт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Продления, шт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка новые, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка продления, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ВЫРУЧКА ИТОГО, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Активные клиенты (оценка)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Эквайринг, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ИИ-затраты, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ВАЛОВАЯ ПРИБЫЛЬ, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Команда, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маркетинг, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Инфраструктура и прочее, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Денежная позиция (раунд + накопл. EBITDA), $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Активные клиенты ≈ сумма новых за последние 3 месяца (средняя длительность сопровождения ~10 недель). Продления учитываются со сдвигом в 2 месяца.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Годовые итоги и юнит-экономика</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Год 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Год 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Валовая прибыль, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Валовая маржа, %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA-маржа, %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Новых клиентов за год</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Денежная позиция на конец года, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ЮНИТ-ЭКОНОМИКА (на одного клиента)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Средний чек, $</t>
   </si>
   <si>
-    <t xml:space="preserve">Средневзвешенный чек. Формула.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Доля клиентов, продлевающих сопровождение</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — доля повторных покупок после завершения тарифа.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">РОСТ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рост новых клиентов, % в месяц (базовый сценарий)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Базовый: +8% в месяц. Сценарии — на листе «Сценарии».</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ЗАТРАТЫ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Эквайринг Stripe, % от выручки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,9% + $0,30 за транзакцию ≈ 3,2% при среднем чеке. Тариф Stripe US, июль 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ИИ-затраты на активного клиента в месяц, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Оценка из фактических тарифов Claude/GPT при текущем режиме «Лучший ответ».</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Инфраструктура (Vercel, Supabase Pro, домен), $/мес</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Факт: Supabase Pro $25 + Vercel Pro ~$20 + резерв. Фиксированные.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Команда (Карен, Анна, поддержка), $/мес — год 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — суммарные выплаты команде. Замените реальными.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рост затрат на команду в год 2 (множитель)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ: расширение команды на 2-м году.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маркетинг, % от выручки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — бюджет привлечения.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Юристы, бухгалтерия, прочее, $/мес</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ИНВЕСТИЦИИ И ПРИВЛЕЧЕНИЕ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Запрашиваемый раунд, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — сумма, которую вы просите у инвестора.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Стоимость привлечения клиента (CAC), $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ = маркетинг на клиента. Проверится фактом первых месяцев.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Помесячный прогноз (базовый сценарий)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Показатель</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">М24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Новые клиенты</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Продажи «5 недель», шт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Продажи «15 недель», шт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Продления, шт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Выручка новые, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Выручка продления, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ВЫРУЧКА ИТОГО, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Активные клиенты (оценка)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Эквайринг, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ИИ-затраты, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ВАЛОВАЯ ПРИБЫЛЬ, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Команда, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маркетинг, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Инфраструктура и прочее, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EBITDA, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Денежная позиция (раунд + накопл. EBITDA), $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Активные клиенты ≈ сумма новых за последние 3 месяца (средняя длительность сопровождения ~10 недель). Продления учитываются со сдвигом в 2 месяца.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Годовые итоги и юнит-экономика</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Год 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Год 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Выручка, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Валовая прибыль, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Валовая маржа, %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EBITDA-маржа, %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Новых клиентов за год</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Денежная позиция на конец года, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ЮНИТ-ЭКОНОМИКА (на одного клиента)</t>
-  </si>
-  <si>
     <t xml:space="preserve">LTV (чек × (1 + доля продлений)), $</t>
   </si>
   <si>
@@ -353,7 +377,7 @@
     <t xml:space="preserve">LTV / CAC</t>
   </si>
   <si>
-    <t xml:space="preserve">Переменные затраты на клиента (эквайринг + ИИ ~3 мес), $</t>
+    <t xml:space="preserve">Переменные затраты на клиента (эквайринг + ИИ + подарок), $</t>
   </si>
   <si>
     <t xml:space="preserve">Валовая прибыль на клиента, $</t>
@@ -589,6 +613,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -601,15 +633,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="168" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -921,7 +945,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:B17"/>
+  <dimension ref="B1:B18"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -974,21 +998,21 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2"/>
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="B13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1005,6 +1029,11 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="2" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1023,7 +1052,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -1033,7 +1062,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1041,30 +1070,30 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>480</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">B4/24</f>
         <v>20</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1072,82 +1101,96 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="11" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="B9" s="11" t="n">
-        <v>1500</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B10" s="12" t="n">
-        <v>0.4</v>
+        <v>0.05</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="13" t="n">
-        <f aca="false">B8*(1-B10)+B9*B10</f>
-        <v>960</v>
+        <v>27</v>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>180</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="12" t="n">
-        <v>0.2</v>
+        <v>29</v>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>120</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
+      <c r="A13" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>30</v>
+      <c r="A14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="15" t="n">
+        <f aca="false">(B8*(1+B10)+B11)*(1-B13)+B9*(1+B10)*B13</f>
+        <v>2334</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="12" t="n">
-        <v>0.08</v>
+        <v>35</v>
+      </c>
+      <c r="B15" s="14" t="n">
+        <v>0.2</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1155,114 +1198,133 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B18" s="14" t="n">
-        <v>0.032</v>
+        <v>0.08</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>37</v>
-      </c>
+      <c r="A19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" s="16" t="n">
-        <v>130</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>39</v>
+      <c r="A20" s="6" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" s="11" t="n">
-        <v>8000</v>
+        <v>41</v>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>0.032</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" s="17" t="n">
-        <v>1.5</v>
+        <v>43</v>
+      </c>
+      <c r="B22" s="16" t="n">
+        <v>1</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B23" s="12" t="n">
-        <v>0.15</v>
+        <v>45</v>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>130</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" s="11" t="n">
-        <v>500</v>
+        <v>47</v>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>8000</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5"/>
+      <c r="A25" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" s="17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>48</v>
+      <c r="A26" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B27" s="11" t="n">
+        <v>53</v>
+      </c>
+      <c r="B27" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="13" t="n">
         <v>150000</v>
       </c>
-      <c r="C27" s="9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B28" s="11" t="n">
+      <c r="C30" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>52</v>
+      <c r="C31" s="9" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1290,392 +1352,392 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="L2" s="20" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="M2" s="20" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="N2" s="20" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="O2" s="20" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="P2" s="20" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="Q2" s="20" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="R2" s="20" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="S2" s="20" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="T2" s="20" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="U2" s="20" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="V2" s="20" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="W2" s="20" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="X2" s="20" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="Y2" s="20" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B3" s="10" t="n">
         <f aca="false">Вводные!$B$5</f>
         <v>20</v>
       </c>
       <c r="C3" s="10" t="n">
-        <f aca="false">ROUND(B3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(B3*(1+Вводные!$B$18),1)</f>
         <v>21.6</v>
       </c>
       <c r="D3" s="10" t="n">
-        <f aca="false">ROUND(C3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(C3*(1+Вводные!$B$18),1)</f>
         <v>23.3</v>
       </c>
       <c r="E3" s="10" t="n">
-        <f aca="false">ROUND(D3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(D3*(1+Вводные!$B$18),1)</f>
         <v>25.2</v>
       </c>
       <c r="F3" s="10" t="n">
-        <f aca="false">ROUND(E3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(E3*(1+Вводные!$B$18),1)</f>
         <v>27.2</v>
       </c>
       <c r="G3" s="10" t="n">
-        <f aca="false">ROUND(F3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(F3*(1+Вводные!$B$18),1)</f>
         <v>29.4</v>
       </c>
       <c r="H3" s="10" t="n">
-        <f aca="false">ROUND(G3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(G3*(1+Вводные!$B$18),1)</f>
         <v>31.8</v>
       </c>
       <c r="I3" s="10" t="n">
-        <f aca="false">ROUND(H3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(H3*(1+Вводные!$B$18),1)</f>
         <v>34.3</v>
       </c>
       <c r="J3" s="10" t="n">
-        <f aca="false">ROUND(I3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(I3*(1+Вводные!$B$18),1)</f>
         <v>37</v>
       </c>
       <c r="K3" s="10" t="n">
-        <f aca="false">ROUND(J3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(J3*(1+Вводные!$B$18),1)</f>
         <v>40</v>
       </c>
       <c r="L3" s="10" t="n">
-        <f aca="false">ROUND(K3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(K3*(1+Вводные!$B$18),1)</f>
         <v>43.2</v>
       </c>
       <c r="M3" s="10" t="n">
-        <f aca="false">ROUND(L3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(L3*(1+Вводные!$B$18),1)</f>
         <v>46.7</v>
       </c>
       <c r="N3" s="10" t="n">
-        <f aca="false">ROUND(M3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(M3*(1+Вводные!$B$18),1)</f>
         <v>50.4</v>
       </c>
       <c r="O3" s="10" t="n">
-        <f aca="false">ROUND(N3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(N3*(1+Вводные!$B$18),1)</f>
         <v>54.4</v>
       </c>
       <c r="P3" s="10" t="n">
-        <f aca="false">ROUND(O3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(O3*(1+Вводные!$B$18),1)</f>
         <v>58.8</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <f aca="false">ROUND(P3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(P3*(1+Вводные!$B$18),1)</f>
         <v>63.5</v>
       </c>
       <c r="R3" s="10" t="n">
-        <f aca="false">ROUND(Q3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(Q3*(1+Вводные!$B$18),1)</f>
         <v>68.6</v>
       </c>
       <c r="S3" s="10" t="n">
-        <f aca="false">ROUND(R3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(R3*(1+Вводные!$B$18),1)</f>
         <v>74.1</v>
       </c>
       <c r="T3" s="10" t="n">
-        <f aca="false">ROUND(S3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(S3*(1+Вводные!$B$18),1)</f>
         <v>80</v>
       </c>
       <c r="U3" s="10" t="n">
-        <f aca="false">ROUND(T3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(T3*(1+Вводные!$B$18),1)</f>
         <v>86.4</v>
       </c>
       <c r="V3" s="10" t="n">
-        <f aca="false">ROUND(U3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(U3*(1+Вводные!$B$18),1)</f>
         <v>93.3</v>
       </c>
       <c r="W3" s="10" t="n">
-        <f aca="false">ROUND(V3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(V3*(1+Вводные!$B$18),1)</f>
         <v>100.8</v>
       </c>
       <c r="X3" s="10" t="n">
-        <f aca="false">ROUND(W3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(W3*(1+Вводные!$B$18),1)</f>
         <v>108.9</v>
       </c>
       <c r="Y3" s="10" t="n">
-        <f aca="false">ROUND(X3*(1+Вводные!$B$15),1)</f>
+        <f aca="false">ROUND(X3*(1+Вводные!$B$18),1)</f>
         <v>117.6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B4" s="10" t="n">
-        <f aca="false">B3*(1-Вводные!$B$10)</f>
+        <f aca="false">B3*(1-Вводные!$B$13)</f>
         <v>12</v>
       </c>
       <c r="C4" s="10" t="n">
-        <f aca="false">C3*(1-Вводные!$B$10)</f>
+        <f aca="false">C3*(1-Вводные!$B$13)</f>
         <v>12.96</v>
       </c>
       <c r="D4" s="10" t="n">
-        <f aca="false">D3*(1-Вводные!$B$10)</f>
+        <f aca="false">D3*(1-Вводные!$B$13)</f>
         <v>13.98</v>
       </c>
       <c r="E4" s="10" t="n">
-        <f aca="false">E3*(1-Вводные!$B$10)</f>
+        <f aca="false">E3*(1-Вводные!$B$13)</f>
         <v>15.12</v>
       </c>
       <c r="F4" s="10" t="n">
-        <f aca="false">F3*(1-Вводные!$B$10)</f>
+        <f aca="false">F3*(1-Вводные!$B$13)</f>
         <v>16.32</v>
       </c>
       <c r="G4" s="10" t="n">
-        <f aca="false">G3*(1-Вводные!$B$10)</f>
+        <f aca="false">G3*(1-Вводные!$B$13)</f>
         <v>17.64</v>
       </c>
       <c r="H4" s="10" t="n">
-        <f aca="false">H3*(1-Вводные!$B$10)</f>
+        <f aca="false">H3*(1-Вводные!$B$13)</f>
         <v>19.08</v>
       </c>
       <c r="I4" s="10" t="n">
-        <f aca="false">I3*(1-Вводные!$B$10)</f>
+        <f aca="false">I3*(1-Вводные!$B$13)</f>
         <v>20.58</v>
       </c>
       <c r="J4" s="10" t="n">
-        <f aca="false">J3*(1-Вводные!$B$10)</f>
+        <f aca="false">J3*(1-Вводные!$B$13)</f>
         <v>22.2</v>
       </c>
       <c r="K4" s="10" t="n">
-        <f aca="false">K3*(1-Вводные!$B$10)</f>
+        <f aca="false">K3*(1-Вводные!$B$13)</f>
         <v>24</v>
       </c>
       <c r="L4" s="10" t="n">
-        <f aca="false">L3*(1-Вводные!$B$10)</f>
+        <f aca="false">L3*(1-Вводные!$B$13)</f>
         <v>25.92</v>
       </c>
       <c r="M4" s="10" t="n">
-        <f aca="false">M3*(1-Вводные!$B$10)</f>
+        <f aca="false">M3*(1-Вводные!$B$13)</f>
         <v>28.02</v>
       </c>
       <c r="N4" s="10" t="n">
-        <f aca="false">N3*(1-Вводные!$B$10)</f>
+        <f aca="false">N3*(1-Вводные!$B$13)</f>
         <v>30.24</v>
       </c>
       <c r="O4" s="10" t="n">
-        <f aca="false">O3*(1-Вводные!$B$10)</f>
+        <f aca="false">O3*(1-Вводные!$B$13)</f>
         <v>32.64</v>
       </c>
       <c r="P4" s="10" t="n">
-        <f aca="false">P3*(1-Вводные!$B$10)</f>
+        <f aca="false">P3*(1-Вводные!$B$13)</f>
         <v>35.28</v>
       </c>
       <c r="Q4" s="10" t="n">
-        <f aca="false">Q3*(1-Вводные!$B$10)</f>
+        <f aca="false">Q3*(1-Вводные!$B$13)</f>
         <v>38.1</v>
       </c>
       <c r="R4" s="10" t="n">
-        <f aca="false">R3*(1-Вводные!$B$10)</f>
+        <f aca="false">R3*(1-Вводные!$B$13)</f>
         <v>41.16</v>
       </c>
       <c r="S4" s="10" t="n">
-        <f aca="false">S3*(1-Вводные!$B$10)</f>
+        <f aca="false">S3*(1-Вводные!$B$13)</f>
         <v>44.46</v>
       </c>
       <c r="T4" s="10" t="n">
-        <f aca="false">T3*(1-Вводные!$B$10)</f>
+        <f aca="false">T3*(1-Вводные!$B$13)</f>
         <v>48</v>
       </c>
       <c r="U4" s="10" t="n">
-        <f aca="false">U3*(1-Вводные!$B$10)</f>
+        <f aca="false">U3*(1-Вводные!$B$13)</f>
         <v>51.84</v>
       </c>
       <c r="V4" s="10" t="n">
-        <f aca="false">V3*(1-Вводные!$B$10)</f>
+        <f aca="false">V3*(1-Вводные!$B$13)</f>
         <v>55.98</v>
       </c>
       <c r="W4" s="10" t="n">
-        <f aca="false">W3*(1-Вводные!$B$10)</f>
+        <f aca="false">W3*(1-Вводные!$B$13)</f>
         <v>60.48</v>
       </c>
       <c r="X4" s="10" t="n">
-        <f aca="false">X3*(1-Вводные!$B$10)</f>
+        <f aca="false">X3*(1-Вводные!$B$13)</f>
         <v>65.34</v>
       </c>
       <c r="Y4" s="10" t="n">
-        <f aca="false">Y3*(1-Вводные!$B$10)</f>
+        <f aca="false">Y3*(1-Вводные!$B$13)</f>
         <v>70.56</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B5" s="10" t="n">
-        <f aca="false">B3*Вводные!$B$10</f>
+        <f aca="false">B3*Вводные!$B$13</f>
         <v>8</v>
       </c>
       <c r="C5" s="10" t="n">
-        <f aca="false">C3*Вводные!$B$10</f>
+        <f aca="false">C3*Вводные!$B$13</f>
         <v>8.64</v>
       </c>
       <c r="D5" s="10" t="n">
-        <f aca="false">D3*Вводные!$B$10</f>
+        <f aca="false">D3*Вводные!$B$13</f>
         <v>9.32</v>
       </c>
       <c r="E5" s="10" t="n">
-        <f aca="false">E3*Вводные!$B$10</f>
+        <f aca="false">E3*Вводные!$B$13</f>
         <v>10.08</v>
       </c>
       <c r="F5" s="10" t="n">
-        <f aca="false">F3*Вводные!$B$10</f>
+        <f aca="false">F3*Вводные!$B$13</f>
         <v>10.88</v>
       </c>
       <c r="G5" s="10" t="n">
-        <f aca="false">G3*Вводные!$B$10</f>
+        <f aca="false">G3*Вводные!$B$13</f>
         <v>11.76</v>
       </c>
       <c r="H5" s="10" t="n">
-        <f aca="false">H3*Вводные!$B$10</f>
+        <f aca="false">H3*Вводные!$B$13</f>
         <v>12.72</v>
       </c>
       <c r="I5" s="10" t="n">
-        <f aca="false">I3*Вводные!$B$10</f>
+        <f aca="false">I3*Вводные!$B$13</f>
         <v>13.72</v>
       </c>
       <c r="J5" s="10" t="n">
-        <f aca="false">J3*Вводные!$B$10</f>
+        <f aca="false">J3*Вводные!$B$13</f>
         <v>14.8</v>
       </c>
       <c r="K5" s="10" t="n">
-        <f aca="false">K3*Вводные!$B$10</f>
+        <f aca="false">K3*Вводные!$B$13</f>
         <v>16</v>
       </c>
       <c r="L5" s="10" t="n">
-        <f aca="false">L3*Вводные!$B$10</f>
+        <f aca="false">L3*Вводные!$B$13</f>
         <v>17.28</v>
       </c>
       <c r="M5" s="10" t="n">
-        <f aca="false">M3*Вводные!$B$10</f>
+        <f aca="false">M3*Вводные!$B$13</f>
         <v>18.68</v>
       </c>
       <c r="N5" s="10" t="n">
-        <f aca="false">N3*Вводные!$B$10</f>
+        <f aca="false">N3*Вводные!$B$13</f>
         <v>20.16</v>
       </c>
       <c r="O5" s="10" t="n">
-        <f aca="false">O3*Вводные!$B$10</f>
+        <f aca="false">O3*Вводные!$B$13</f>
         <v>21.76</v>
       </c>
       <c r="P5" s="10" t="n">
-        <f aca="false">P3*Вводные!$B$10</f>
+        <f aca="false">P3*Вводные!$B$13</f>
         <v>23.52</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <f aca="false">Q3*Вводные!$B$10</f>
+        <f aca="false">Q3*Вводные!$B$13</f>
         <v>25.4</v>
       </c>
       <c r="R5" s="10" t="n">
-        <f aca="false">R3*Вводные!$B$10</f>
+        <f aca="false">R3*Вводные!$B$13</f>
         <v>27.44</v>
       </c>
       <c r="S5" s="10" t="n">
-        <f aca="false">S3*Вводные!$B$10</f>
+        <f aca="false">S3*Вводные!$B$13</f>
         <v>29.64</v>
       </c>
       <c r="T5" s="10" t="n">
-        <f aca="false">T3*Вводные!$B$10</f>
+        <f aca="false">T3*Вводные!$B$13</f>
         <v>32</v>
       </c>
       <c r="U5" s="10" t="n">
-        <f aca="false">U3*Вводные!$B$10</f>
+        <f aca="false">U3*Вводные!$B$13</f>
         <v>34.56</v>
       </c>
       <c r="V5" s="10" t="n">
-        <f aca="false">V3*Вводные!$B$10</f>
+        <f aca="false">V3*Вводные!$B$13</f>
         <v>37.32</v>
       </c>
       <c r="W5" s="10" t="n">
-        <f aca="false">W3*Вводные!$B$10</f>
+        <f aca="false">W3*Вводные!$B$13</f>
         <v>40.32</v>
       </c>
       <c r="X5" s="10" t="n">
-        <f aca="false">X3*Вводные!$B$10</f>
+        <f aca="false">X3*Вводные!$B$13</f>
         <v>43.56</v>
       </c>
       <c r="Y5" s="10" t="n">
-        <f aca="false">Y3*Вводные!$B$10</f>
+        <f aca="false">Y3*Вводные!$B$13</f>
         <v>47.04</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>0</v>
@@ -1684,401 +1746,401 @@
         <v>0</v>
       </c>
       <c r="D6" s="10" t="n">
-        <f aca="false">B3*Вводные!$B$12</f>
+        <f aca="false">B3*Вводные!$B$15</f>
         <v>4</v>
       </c>
       <c r="E6" s="10" t="n">
-        <f aca="false">C3*Вводные!$B$12</f>
+        <f aca="false">C3*Вводные!$B$15</f>
         <v>4.32</v>
       </c>
       <c r="F6" s="10" t="n">
-        <f aca="false">D3*Вводные!$B$12</f>
+        <f aca="false">D3*Вводные!$B$15</f>
         <v>4.66</v>
       </c>
       <c r="G6" s="10" t="n">
-        <f aca="false">E3*Вводные!$B$12</f>
+        <f aca="false">E3*Вводные!$B$15</f>
         <v>5.04</v>
       </c>
       <c r="H6" s="10" t="n">
-        <f aca="false">F3*Вводные!$B$12</f>
+        <f aca="false">F3*Вводные!$B$15</f>
         <v>5.44</v>
       </c>
       <c r="I6" s="10" t="n">
-        <f aca="false">G3*Вводные!$B$12</f>
+        <f aca="false">G3*Вводные!$B$15</f>
         <v>5.88</v>
       </c>
       <c r="J6" s="10" t="n">
-        <f aca="false">H3*Вводные!$B$12</f>
+        <f aca="false">H3*Вводные!$B$15</f>
         <v>6.36</v>
       </c>
       <c r="K6" s="10" t="n">
-        <f aca="false">I3*Вводные!$B$12</f>
+        <f aca="false">I3*Вводные!$B$15</f>
         <v>6.86</v>
       </c>
       <c r="L6" s="10" t="n">
-        <f aca="false">J3*Вводные!$B$12</f>
+        <f aca="false">J3*Вводные!$B$15</f>
         <v>7.4</v>
       </c>
       <c r="M6" s="10" t="n">
-        <f aca="false">K3*Вводные!$B$12</f>
+        <f aca="false">K3*Вводные!$B$15</f>
         <v>8</v>
       </c>
       <c r="N6" s="10" t="n">
-        <f aca="false">L3*Вводные!$B$12</f>
+        <f aca="false">L3*Вводные!$B$15</f>
         <v>8.64</v>
       </c>
       <c r="O6" s="10" t="n">
-        <f aca="false">M3*Вводные!$B$12</f>
+        <f aca="false">M3*Вводные!$B$15</f>
         <v>9.34</v>
       </c>
       <c r="P6" s="10" t="n">
-        <f aca="false">N3*Вводные!$B$12</f>
+        <f aca="false">N3*Вводные!$B$15</f>
         <v>10.08</v>
       </c>
       <c r="Q6" s="10" t="n">
-        <f aca="false">O3*Вводные!$B$12</f>
+        <f aca="false">O3*Вводные!$B$15</f>
         <v>10.88</v>
       </c>
       <c r="R6" s="10" t="n">
-        <f aca="false">P3*Вводные!$B$12</f>
+        <f aca="false">P3*Вводные!$B$15</f>
         <v>11.76</v>
       </c>
       <c r="S6" s="10" t="n">
-        <f aca="false">Q3*Вводные!$B$12</f>
+        <f aca="false">Q3*Вводные!$B$15</f>
         <v>12.7</v>
       </c>
       <c r="T6" s="10" t="n">
-        <f aca="false">R3*Вводные!$B$12</f>
+        <f aca="false">R3*Вводные!$B$15</f>
         <v>13.72</v>
       </c>
       <c r="U6" s="10" t="n">
-        <f aca="false">S3*Вводные!$B$12</f>
+        <f aca="false">S3*Вводные!$B$15</f>
         <v>14.82</v>
       </c>
       <c r="V6" s="10" t="n">
-        <f aca="false">T3*Вводные!$B$12</f>
+        <f aca="false">T3*Вводные!$B$15</f>
         <v>16</v>
       </c>
       <c r="W6" s="10" t="n">
-        <f aca="false">U3*Вводные!$B$12</f>
+        <f aca="false">U3*Вводные!$B$15</f>
         <v>17.28</v>
       </c>
       <c r="X6" s="10" t="n">
-        <f aca="false">V3*Вводные!$B$12</f>
+        <f aca="false">V3*Вводные!$B$15</f>
         <v>18.66</v>
       </c>
       <c r="Y6" s="10" t="n">
-        <f aca="false">W3*Вводные!$B$12</f>
+        <f aca="false">W3*Вводные!$B$15</f>
         <v>20.16</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="13" t="n">
-        <f aca="false">B4*Вводные!$B$8+B5*Вводные!$B$9</f>
-        <v>19200</v>
-      </c>
-      <c r="C7" s="13" t="n">
-        <f aca="false">C4*Вводные!$B$8+C5*Вводные!$B$9</f>
-        <v>20736</v>
-      </c>
-      <c r="D7" s="13" t="n">
-        <f aca="false">D4*Вводные!$B$8+D5*Вводные!$B$9</f>
-        <v>22368</v>
-      </c>
-      <c r="E7" s="13" t="n">
-        <f aca="false">E4*Вводные!$B$8+E5*Вводные!$B$9</f>
-        <v>24192</v>
-      </c>
-      <c r="F7" s="13" t="n">
-        <f aca="false">F4*Вводные!$B$8+F5*Вводные!$B$9</f>
-        <v>26112</v>
-      </c>
-      <c r="G7" s="13" t="n">
-        <f aca="false">G4*Вводные!$B$8+G5*Вводные!$B$9</f>
-        <v>28224</v>
-      </c>
-      <c r="H7" s="13" t="n">
-        <f aca="false">H4*Вводные!$B$8+H5*Вводные!$B$9</f>
-        <v>30528</v>
-      </c>
-      <c r="I7" s="13" t="n">
-        <f aca="false">I4*Вводные!$B$8+I5*Вводные!$B$9</f>
-        <v>32928</v>
-      </c>
-      <c r="J7" s="13" t="n">
-        <f aca="false">J4*Вводные!$B$8+J5*Вводные!$B$9</f>
-        <v>35520</v>
-      </c>
-      <c r="K7" s="13" t="n">
-        <f aca="false">K4*Вводные!$B$8+K5*Вводные!$B$9</f>
-        <v>38400</v>
-      </c>
-      <c r="L7" s="13" t="n">
-        <f aca="false">L4*Вводные!$B$8+L5*Вводные!$B$9</f>
-        <v>41472</v>
-      </c>
-      <c r="M7" s="13" t="n">
-        <f aca="false">M4*Вводные!$B$8+M5*Вводные!$B$9</f>
-        <v>44832</v>
-      </c>
-      <c r="N7" s="13" t="n">
-        <f aca="false">N4*Вводные!$B$8+N5*Вводные!$B$9</f>
-        <v>48384</v>
-      </c>
-      <c r="O7" s="13" t="n">
-        <f aca="false">O4*Вводные!$B$8+O5*Вводные!$B$9</f>
-        <v>52224</v>
-      </c>
-      <c r="P7" s="13" t="n">
-        <f aca="false">P4*Вводные!$B$8+P5*Вводные!$B$9</f>
-        <v>56448</v>
-      </c>
-      <c r="Q7" s="13" t="n">
-        <f aca="false">Q4*Вводные!$B$8+Q5*Вводные!$B$9</f>
-        <v>60960</v>
-      </c>
-      <c r="R7" s="13" t="n">
-        <f aca="false">R4*Вводные!$B$8+R5*Вводные!$B$9</f>
-        <v>65856</v>
-      </c>
-      <c r="S7" s="13" t="n">
-        <f aca="false">S4*Вводные!$B$8+S5*Вводные!$B$9</f>
-        <v>71136</v>
-      </c>
-      <c r="T7" s="13" t="n">
-        <f aca="false">T4*Вводные!$B$8+T5*Вводные!$B$9</f>
-        <v>76800</v>
-      </c>
-      <c r="U7" s="13" t="n">
-        <f aca="false">U4*Вводные!$B$8+U5*Вводные!$B$9</f>
-        <v>82944</v>
-      </c>
-      <c r="V7" s="13" t="n">
-        <f aca="false">V4*Вводные!$B$8+V5*Вводные!$B$9</f>
-        <v>89568</v>
-      </c>
-      <c r="W7" s="13" t="n">
-        <f aca="false">W4*Вводные!$B$8+W5*Вводные!$B$9</f>
-        <v>96768</v>
-      </c>
-      <c r="X7" s="13" t="n">
-        <f aca="false">X4*Вводные!$B$8+X5*Вводные!$B$9</f>
-        <v>104544</v>
-      </c>
-      <c r="Y7" s="13" t="n">
-        <f aca="false">Y4*Вводные!$B$8+Y5*Вводные!$B$9</f>
-        <v>112896</v>
+        <v>90</v>
+      </c>
+      <c r="B7" s="15" t="n">
+        <f aca="false">B4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+B5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>46680</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <f aca="false">C4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+C5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>50414.4</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <f aca="false">D4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+D5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>54382.2</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <f aca="false">E4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+E5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>58816.8</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <f aca="false">F4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+F5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>63484.8</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <f aca="false">G4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+G5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>68619.6</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <f aca="false">H4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+H5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>74221.2</v>
+      </c>
+      <c r="I7" s="15" t="n">
+        <f aca="false">I4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+I5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>80056.2</v>
+      </c>
+      <c r="J7" s="15" t="n">
+        <f aca="false">J4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+J5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>86358</v>
+      </c>
+      <c r="K7" s="15" t="n">
+        <f aca="false">K4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+K5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>93360</v>
+      </c>
+      <c r="L7" s="15" t="n">
+        <f aca="false">L4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+L5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>100828.8</v>
+      </c>
+      <c r="M7" s="15" t="n">
+        <f aca="false">M4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+M5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>108997.8</v>
+      </c>
+      <c r="N7" s="15" t="n">
+        <f aca="false">N4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+N5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>117633.6</v>
+      </c>
+      <c r="O7" s="15" t="n">
+        <f aca="false">O4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+O5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>126969.6</v>
+      </c>
+      <c r="P7" s="15" t="n">
+        <f aca="false">P4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+P5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>137239.2</v>
+      </c>
+      <c r="Q7" s="15" t="n">
+        <f aca="false">Q4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+Q5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>148209</v>
+      </c>
+      <c r="R7" s="15" t="n">
+        <f aca="false">R4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+R5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>160112.4</v>
+      </c>
+      <c r="S7" s="15" t="n">
+        <f aca="false">S4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+S5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>172949.4</v>
+      </c>
+      <c r="T7" s="15" t="n">
+        <f aca="false">T4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+T5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>186720</v>
+      </c>
+      <c r="U7" s="15" t="n">
+        <f aca="false">U4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+U5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>201657.6</v>
+      </c>
+      <c r="V7" s="15" t="n">
+        <f aca="false">V4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+V5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>217762.2</v>
+      </c>
+      <c r="W7" s="15" t="n">
+        <f aca="false">W4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+W5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>235267.2</v>
+      </c>
+      <c r="X7" s="15" t="n">
+        <f aca="false">X4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+X5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>254172.6</v>
+      </c>
+      <c r="Y7" s="15" t="n">
+        <f aca="false">Y4*(Вводные!$B$8*(1+Вводные!$B$10)+Вводные!$B$11)+Y5*Вводные!$B$9*(1+Вводные!$B$10)</f>
+        <v>274478.4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" s="13" t="n">
-        <f aca="false">B6*Вводные!$B$11</f>
+        <v>91</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <f aca="false">B6*Вводные!$B$14</f>
         <v>0</v>
       </c>
-      <c r="C8" s="13" t="n">
-        <f aca="false">C6*Вводные!$B$11</f>
+      <c r="C8" s="15" t="n">
+        <f aca="false">C6*Вводные!$B$14</f>
         <v>0</v>
       </c>
-      <c r="D8" s="13" t="n">
-        <f aca="false">D6*Вводные!$B$11</f>
-        <v>3840</v>
-      </c>
-      <c r="E8" s="13" t="n">
-        <f aca="false">E6*Вводные!$B$11</f>
-        <v>4147.2</v>
-      </c>
-      <c r="F8" s="13" t="n">
-        <f aca="false">F6*Вводные!$B$11</f>
-        <v>4473.6</v>
-      </c>
-      <c r="G8" s="13" t="n">
-        <f aca="false">G6*Вводные!$B$11</f>
-        <v>4838.4</v>
-      </c>
-      <c r="H8" s="13" t="n">
-        <f aca="false">H6*Вводные!$B$11</f>
-        <v>5222.4</v>
-      </c>
-      <c r="I8" s="13" t="n">
-        <f aca="false">I6*Вводные!$B$11</f>
-        <v>5644.8</v>
-      </c>
-      <c r="J8" s="13" t="n">
-        <f aca="false">J6*Вводные!$B$11</f>
-        <v>6105.6</v>
-      </c>
-      <c r="K8" s="13" t="n">
-        <f aca="false">K6*Вводные!$B$11</f>
-        <v>6585.6</v>
-      </c>
-      <c r="L8" s="13" t="n">
-        <f aca="false">L6*Вводные!$B$11</f>
-        <v>7104</v>
-      </c>
-      <c r="M8" s="13" t="n">
-        <f aca="false">M6*Вводные!$B$11</f>
-        <v>7680</v>
-      </c>
-      <c r="N8" s="13" t="n">
-        <f aca="false">N6*Вводные!$B$11</f>
-        <v>8294.4</v>
-      </c>
-      <c r="O8" s="13" t="n">
-        <f aca="false">O6*Вводные!$B$11</f>
-        <v>8966.4</v>
-      </c>
-      <c r="P8" s="13" t="n">
-        <f aca="false">P6*Вводные!$B$11</f>
-        <v>9676.8</v>
-      </c>
-      <c r="Q8" s="13" t="n">
-        <f aca="false">Q6*Вводные!$B$11</f>
-        <v>10444.8</v>
-      </c>
-      <c r="R8" s="13" t="n">
-        <f aca="false">R6*Вводные!$B$11</f>
-        <v>11289.6</v>
-      </c>
-      <c r="S8" s="13" t="n">
-        <f aca="false">S6*Вводные!$B$11</f>
-        <v>12192</v>
-      </c>
-      <c r="T8" s="13" t="n">
-        <f aca="false">T6*Вводные!$B$11</f>
-        <v>13171.2</v>
-      </c>
-      <c r="U8" s="13" t="n">
-        <f aca="false">U6*Вводные!$B$11</f>
-        <v>14227.2</v>
-      </c>
-      <c r="V8" s="13" t="n">
-        <f aca="false">V6*Вводные!$B$11</f>
-        <v>15360</v>
-      </c>
-      <c r="W8" s="13" t="n">
-        <f aca="false">W6*Вводные!$B$11</f>
-        <v>16588.8</v>
-      </c>
-      <c r="X8" s="13" t="n">
-        <f aca="false">X6*Вводные!$B$11</f>
-        <v>17913.6</v>
-      </c>
-      <c r="Y8" s="13" t="n">
-        <f aca="false">Y6*Вводные!$B$11</f>
-        <v>19353.6</v>
+      <c r="D8" s="15" t="n">
+        <f aca="false">D6*Вводные!$B$14</f>
+        <v>9336</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <f aca="false">E6*Вводные!$B$14</f>
+        <v>10082.88</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <f aca="false">F6*Вводные!$B$14</f>
+        <v>10876.44</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <f aca="false">G6*Вводные!$B$14</f>
+        <v>11763.36</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <f aca="false">H6*Вводные!$B$14</f>
+        <v>12696.96</v>
+      </c>
+      <c r="I8" s="15" t="n">
+        <f aca="false">I6*Вводные!$B$14</f>
+        <v>13723.92</v>
+      </c>
+      <c r="J8" s="15" t="n">
+        <f aca="false">J6*Вводные!$B$14</f>
+        <v>14844.24</v>
+      </c>
+      <c r="K8" s="15" t="n">
+        <f aca="false">K6*Вводные!$B$14</f>
+        <v>16011.24</v>
+      </c>
+      <c r="L8" s="15" t="n">
+        <f aca="false">L6*Вводные!$B$14</f>
+        <v>17271.6</v>
+      </c>
+      <c r="M8" s="15" t="n">
+        <f aca="false">M6*Вводные!$B$14</f>
+        <v>18672</v>
+      </c>
+      <c r="N8" s="15" t="n">
+        <f aca="false">N6*Вводные!$B$14</f>
+        <v>20165.76</v>
+      </c>
+      <c r="O8" s="15" t="n">
+        <f aca="false">O6*Вводные!$B$14</f>
+        <v>21799.56</v>
+      </c>
+      <c r="P8" s="15" t="n">
+        <f aca="false">P6*Вводные!$B$14</f>
+        <v>23526.72</v>
+      </c>
+      <c r="Q8" s="15" t="n">
+        <f aca="false">Q6*Вводные!$B$14</f>
+        <v>25393.92</v>
+      </c>
+      <c r="R8" s="15" t="n">
+        <f aca="false">R6*Вводные!$B$14</f>
+        <v>27447.84</v>
+      </c>
+      <c r="S8" s="15" t="n">
+        <f aca="false">S6*Вводные!$B$14</f>
+        <v>29641.8</v>
+      </c>
+      <c r="T8" s="15" t="n">
+        <f aca="false">T6*Вводные!$B$14</f>
+        <v>32022.48</v>
+      </c>
+      <c r="U8" s="15" t="n">
+        <f aca="false">U6*Вводные!$B$14</f>
+        <v>34589.88</v>
+      </c>
+      <c r="V8" s="15" t="n">
+        <f aca="false">V6*Вводные!$B$14</f>
+        <v>37344</v>
+      </c>
+      <c r="W8" s="15" t="n">
+        <f aca="false">W6*Вводные!$B$14</f>
+        <v>40331.52</v>
+      </c>
+      <c r="X8" s="15" t="n">
+        <f aca="false">X6*Вводные!$B$14</f>
+        <v>43552.44</v>
+      </c>
+      <c r="Y8" s="15" t="n">
+        <f aca="false">Y6*Вводные!$B$14</f>
+        <v>47053.44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B9" s="23" t="n">
         <f aca="false">B7+B8</f>
-        <v>19200</v>
+        <v>46680</v>
       </c>
       <c r="C9" s="23" t="n">
         <f aca="false">C7+C8</f>
-        <v>20736</v>
+        <v>50414.4</v>
       </c>
       <c r="D9" s="23" t="n">
         <f aca="false">D7+D8</f>
-        <v>26208</v>
+        <v>63718.2</v>
       </c>
       <c r="E9" s="23" t="n">
         <f aca="false">E7+E8</f>
-        <v>28339.2</v>
+        <v>68899.68</v>
       </c>
       <c r="F9" s="23" t="n">
         <f aca="false">F7+F8</f>
-        <v>30585.6</v>
+        <v>74361.24</v>
       </c>
       <c r="G9" s="23" t="n">
         <f aca="false">G7+G8</f>
-        <v>33062.4</v>
+        <v>80382.96</v>
       </c>
       <c r="H9" s="23" t="n">
         <f aca="false">H7+H8</f>
-        <v>35750.4</v>
+        <v>86918.16</v>
       </c>
       <c r="I9" s="23" t="n">
         <f aca="false">I7+I8</f>
-        <v>38572.8</v>
+        <v>93780.12</v>
       </c>
       <c r="J9" s="23" t="n">
         <f aca="false">J7+J8</f>
-        <v>41625.6</v>
+        <v>101202.24</v>
       </c>
       <c r="K9" s="23" t="n">
         <f aca="false">K7+K8</f>
-        <v>44985.6</v>
+        <v>109371.24</v>
       </c>
       <c r="L9" s="23" t="n">
         <f aca="false">L7+L8</f>
-        <v>48576</v>
+        <v>118100.4</v>
       </c>
       <c r="M9" s="23" t="n">
         <f aca="false">M7+M8</f>
-        <v>52512</v>
+        <v>127669.8</v>
       </c>
       <c r="N9" s="23" t="n">
         <f aca="false">N7+N8</f>
-        <v>56678.4</v>
+        <v>137799.36</v>
       </c>
       <c r="O9" s="23" t="n">
         <f aca="false">O7+O8</f>
-        <v>61190.4</v>
+        <v>148769.16</v>
       </c>
       <c r="P9" s="23" t="n">
         <f aca="false">P7+P8</f>
-        <v>66124.8</v>
+        <v>160765.92</v>
       </c>
       <c r="Q9" s="23" t="n">
         <f aca="false">Q7+Q8</f>
-        <v>71404.8</v>
+        <v>173602.92</v>
       </c>
       <c r="R9" s="23" t="n">
         <f aca="false">R7+R8</f>
-        <v>77145.6</v>
+        <v>187560.24</v>
       </c>
       <c r="S9" s="23" t="n">
         <f aca="false">S7+S8</f>
-        <v>83328</v>
+        <v>202591.2</v>
       </c>
       <c r="T9" s="23" t="n">
         <f aca="false">T7+T8</f>
-        <v>89971.2</v>
+        <v>218742.48</v>
       </c>
       <c r="U9" s="23" t="n">
         <f aca="false">U7+U8</f>
-        <v>97171.2</v>
+        <v>236247.48</v>
       </c>
       <c r="V9" s="23" t="n">
         <f aca="false">V7+V8</f>
-        <v>104928</v>
+        <v>255106.2</v>
       </c>
       <c r="W9" s="23" t="n">
         <f aca="false">W7+W8</f>
-        <v>113356.8</v>
+        <v>275598.72</v>
       </c>
       <c r="X9" s="23" t="n">
         <f aca="false">X7+X8</f>
-        <v>122457.6</v>
+        <v>297725.04</v>
       </c>
       <c r="Y9" s="23" t="n">
         <f aca="false">Y7+Y8</f>
-        <v>132249.6</v>
+        <v>321531.84</v>
       </c>
       <c r="Z9" s="24"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B10" s="10" t="n">
         <f aca="false">B3</f>
@@ -2179,818 +2241,818 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="B11" s="13" t="n">
-        <f aca="false">B9*Вводные!$B$18</f>
-        <v>614.4</v>
-      </c>
-      <c r="C11" s="13" t="n">
-        <f aca="false">C9*Вводные!$B$18</f>
-        <v>663.552</v>
-      </c>
-      <c r="D11" s="13" t="n">
-        <f aca="false">D9*Вводные!$B$18</f>
-        <v>838.656</v>
-      </c>
-      <c r="E11" s="13" t="n">
-        <f aca="false">E9*Вводные!$B$18</f>
-        <v>906.8544</v>
-      </c>
-      <c r="F11" s="13" t="n">
-        <f aca="false">F9*Вводные!$B$18</f>
-        <v>978.7392</v>
-      </c>
-      <c r="G11" s="13" t="n">
-        <f aca="false">G9*Вводные!$B$18</f>
-        <v>1057.9968</v>
-      </c>
-      <c r="H11" s="13" t="n">
-        <f aca="false">H9*Вводные!$B$18</f>
-        <v>1144.0128</v>
-      </c>
-      <c r="I11" s="13" t="n">
-        <f aca="false">I9*Вводные!$B$18</f>
-        <v>1234.3296</v>
-      </c>
-      <c r="J11" s="13" t="n">
-        <f aca="false">J9*Вводные!$B$18</f>
-        <v>1332.0192</v>
-      </c>
-      <c r="K11" s="13" t="n">
-        <f aca="false">K9*Вводные!$B$18</f>
-        <v>1439.5392</v>
-      </c>
-      <c r="L11" s="13" t="n">
-        <f aca="false">L9*Вводные!$B$18</f>
-        <v>1554.432</v>
-      </c>
-      <c r="M11" s="13" t="n">
-        <f aca="false">M9*Вводные!$B$18</f>
-        <v>1680.384</v>
-      </c>
-      <c r="N11" s="13" t="n">
-        <f aca="false">N9*Вводные!$B$18</f>
-        <v>1813.7088</v>
-      </c>
-      <c r="O11" s="13" t="n">
-        <f aca="false">O9*Вводные!$B$18</f>
-        <v>1958.0928</v>
-      </c>
-      <c r="P11" s="13" t="n">
-        <f aca="false">P9*Вводные!$B$18</f>
-        <v>2115.9936</v>
-      </c>
-      <c r="Q11" s="13" t="n">
-        <f aca="false">Q9*Вводные!$B$18</f>
-        <v>2284.9536</v>
-      </c>
-      <c r="R11" s="13" t="n">
-        <f aca="false">R9*Вводные!$B$18</f>
-        <v>2468.6592</v>
-      </c>
-      <c r="S11" s="13" t="n">
-        <f aca="false">S9*Вводные!$B$18</f>
-        <v>2666.496</v>
-      </c>
-      <c r="T11" s="13" t="n">
-        <f aca="false">T9*Вводные!$B$18</f>
-        <v>2879.0784</v>
-      </c>
-      <c r="U11" s="13" t="n">
-        <f aca="false">U9*Вводные!$B$18</f>
-        <v>3109.4784</v>
-      </c>
-      <c r="V11" s="13" t="n">
-        <f aca="false">V9*Вводные!$B$18</f>
-        <v>3357.696</v>
-      </c>
-      <c r="W11" s="13" t="n">
-        <f aca="false">W9*Вводные!$B$18</f>
-        <v>3627.4176</v>
-      </c>
-      <c r="X11" s="13" t="n">
-        <f aca="false">X9*Вводные!$B$18</f>
-        <v>3918.6432</v>
-      </c>
-      <c r="Y11" s="13" t="n">
-        <f aca="false">Y9*Вводные!$B$18</f>
-        <v>4231.9872</v>
+        <v>94</v>
+      </c>
+      <c r="B11" s="15" t="n">
+        <f aca="false">B9*Вводные!$B$21</f>
+        <v>1493.76</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <f aca="false">C9*Вводные!$B$21</f>
+        <v>1613.2608</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <f aca="false">D9*Вводные!$B$21</f>
+        <v>2038.9824</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <f aca="false">E9*Вводные!$B$21</f>
+        <v>2204.78976</v>
+      </c>
+      <c r="F11" s="15" t="n">
+        <f aca="false">F9*Вводные!$B$21</f>
+        <v>2379.55968</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <f aca="false">G9*Вводные!$B$21</f>
+        <v>2572.25472</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <f aca="false">H9*Вводные!$B$21</f>
+        <v>2781.38112</v>
+      </c>
+      <c r="I11" s="15" t="n">
+        <f aca="false">I9*Вводные!$B$21</f>
+        <v>3000.96384</v>
+      </c>
+      <c r="J11" s="15" t="n">
+        <f aca="false">J9*Вводные!$B$21</f>
+        <v>3238.47168</v>
+      </c>
+      <c r="K11" s="15" t="n">
+        <f aca="false">K9*Вводные!$B$21</f>
+        <v>3499.87968</v>
+      </c>
+      <c r="L11" s="15" t="n">
+        <f aca="false">L9*Вводные!$B$21</f>
+        <v>3779.2128</v>
+      </c>
+      <c r="M11" s="15" t="n">
+        <f aca="false">M9*Вводные!$B$21</f>
+        <v>4085.4336</v>
+      </c>
+      <c r="N11" s="15" t="n">
+        <f aca="false">N9*Вводные!$B$21</f>
+        <v>4409.57952</v>
+      </c>
+      <c r="O11" s="15" t="n">
+        <f aca="false">O9*Вводные!$B$21</f>
+        <v>4760.61312</v>
+      </c>
+      <c r="P11" s="15" t="n">
+        <f aca="false">P9*Вводные!$B$21</f>
+        <v>5144.50944</v>
+      </c>
+      <c r="Q11" s="15" t="n">
+        <f aca="false">Q9*Вводные!$B$21</f>
+        <v>5555.29344</v>
+      </c>
+      <c r="R11" s="15" t="n">
+        <f aca="false">R9*Вводные!$B$21</f>
+        <v>6001.92768</v>
+      </c>
+      <c r="S11" s="15" t="n">
+        <f aca="false">S9*Вводные!$B$21</f>
+        <v>6482.9184</v>
+      </c>
+      <c r="T11" s="15" t="n">
+        <f aca="false">T9*Вводные!$B$21</f>
+        <v>6999.75936</v>
+      </c>
+      <c r="U11" s="15" t="n">
+        <f aca="false">U9*Вводные!$B$21</f>
+        <v>7559.91936</v>
+      </c>
+      <c r="V11" s="15" t="n">
+        <f aca="false">V9*Вводные!$B$21</f>
+        <v>8163.3984</v>
+      </c>
+      <c r="W11" s="15" t="n">
+        <f aca="false">W9*Вводные!$B$21</f>
+        <v>8819.15904</v>
+      </c>
+      <c r="X11" s="15" t="n">
+        <f aca="false">X9*Вводные!$B$21</f>
+        <v>9527.20128</v>
+      </c>
+      <c r="Y11" s="15" t="n">
+        <f aca="false">Y9*Вводные!$B$21</f>
+        <v>10289.01888</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="13" t="n">
-        <f aca="false">B10*Вводные!$B$19</f>
+        <v>95</v>
+      </c>
+      <c r="B12" s="15" t="n">
+        <f aca="false">B10*Вводные!$B$22</f>
         <v>20</v>
       </c>
-      <c r="C12" s="13" t="n">
-        <f aca="false">C10*Вводные!$B$19</f>
+      <c r="C12" s="15" t="n">
+        <f aca="false">C10*Вводные!$B$22</f>
         <v>41.6</v>
       </c>
-      <c r="D12" s="13" t="n">
-        <f aca="false">D10*Вводные!$B$19</f>
+      <c r="D12" s="15" t="n">
+        <f aca="false">D10*Вводные!$B$22</f>
         <v>64.9</v>
       </c>
-      <c r="E12" s="13" t="n">
-        <f aca="false">E10*Вводные!$B$19</f>
+      <c r="E12" s="15" t="n">
+        <f aca="false">E10*Вводные!$B$22</f>
         <v>70.1</v>
       </c>
-      <c r="F12" s="13" t="n">
-        <f aca="false">F10*Вводные!$B$19</f>
+      <c r="F12" s="15" t="n">
+        <f aca="false">F10*Вводные!$B$22</f>
         <v>75.7</v>
       </c>
-      <c r="G12" s="13" t="n">
-        <f aca="false">G10*Вводные!$B$19</f>
+      <c r="G12" s="15" t="n">
+        <f aca="false">G10*Вводные!$B$22</f>
         <v>81.8</v>
       </c>
-      <c r="H12" s="13" t="n">
-        <f aca="false">H10*Вводные!$B$19</f>
+      <c r="H12" s="15" t="n">
+        <f aca="false">H10*Вводные!$B$22</f>
         <v>88.4</v>
       </c>
-      <c r="I12" s="13" t="n">
-        <f aca="false">I10*Вводные!$B$19</f>
+      <c r="I12" s="15" t="n">
+        <f aca="false">I10*Вводные!$B$22</f>
         <v>95.5</v>
       </c>
-      <c r="J12" s="13" t="n">
-        <f aca="false">J10*Вводные!$B$19</f>
+      <c r="J12" s="15" t="n">
+        <f aca="false">J10*Вводные!$B$22</f>
         <v>103.1</v>
       </c>
-      <c r="K12" s="13" t="n">
-        <f aca="false">K10*Вводные!$B$19</f>
+      <c r="K12" s="15" t="n">
+        <f aca="false">K10*Вводные!$B$22</f>
         <v>111.3</v>
       </c>
-      <c r="L12" s="13" t="n">
-        <f aca="false">L10*Вводные!$B$19</f>
+      <c r="L12" s="15" t="n">
+        <f aca="false">L10*Вводные!$B$22</f>
         <v>120.2</v>
       </c>
-      <c r="M12" s="13" t="n">
-        <f aca="false">M10*Вводные!$B$19</f>
+      <c r="M12" s="15" t="n">
+        <f aca="false">M10*Вводные!$B$22</f>
         <v>129.9</v>
       </c>
-      <c r="N12" s="13" t="n">
-        <f aca="false">N10*Вводные!$B$19</f>
+      <c r="N12" s="15" t="n">
+        <f aca="false">N10*Вводные!$B$22</f>
         <v>140.3</v>
       </c>
-      <c r="O12" s="13" t="n">
-        <f aca="false">O10*Вводные!$B$19</f>
+      <c r="O12" s="15" t="n">
+        <f aca="false">O10*Вводные!$B$22</f>
         <v>151.5</v>
       </c>
-      <c r="P12" s="13" t="n">
-        <f aca="false">P10*Вводные!$B$19</f>
+      <c r="P12" s="15" t="n">
+        <f aca="false">P10*Вводные!$B$22</f>
         <v>163.6</v>
       </c>
-      <c r="Q12" s="13" t="n">
-        <f aca="false">Q10*Вводные!$B$19</f>
+      <c r="Q12" s="15" t="n">
+        <f aca="false">Q10*Вводные!$B$22</f>
         <v>176.7</v>
       </c>
-      <c r="R12" s="13" t="n">
-        <f aca="false">R10*Вводные!$B$19</f>
+      <c r="R12" s="15" t="n">
+        <f aca="false">R10*Вводные!$B$22</f>
         <v>190.9</v>
       </c>
-      <c r="S12" s="13" t="n">
-        <f aca="false">S10*Вводные!$B$19</f>
+      <c r="S12" s="15" t="n">
+        <f aca="false">S10*Вводные!$B$22</f>
         <v>206.2</v>
       </c>
-      <c r="T12" s="13" t="n">
-        <f aca="false">T10*Вводные!$B$19</f>
+      <c r="T12" s="15" t="n">
+        <f aca="false">T10*Вводные!$B$22</f>
         <v>222.7</v>
       </c>
-      <c r="U12" s="13" t="n">
-        <f aca="false">U10*Вводные!$B$19</f>
+      <c r="U12" s="15" t="n">
+        <f aca="false">U10*Вводные!$B$22</f>
         <v>240.5</v>
       </c>
-      <c r="V12" s="13" t="n">
-        <f aca="false">V10*Вводные!$B$19</f>
+      <c r="V12" s="15" t="n">
+        <f aca="false">V10*Вводные!$B$22</f>
         <v>259.7</v>
       </c>
-      <c r="W12" s="13" t="n">
-        <f aca="false">W10*Вводные!$B$19</f>
+      <c r="W12" s="15" t="n">
+        <f aca="false">W10*Вводные!$B$22</f>
         <v>280.5</v>
       </c>
-      <c r="X12" s="13" t="n">
-        <f aca="false">X10*Вводные!$B$19</f>
+      <c r="X12" s="15" t="n">
+        <f aca="false">X10*Вводные!$B$22</f>
         <v>303</v>
       </c>
-      <c r="Y12" s="13" t="n">
-        <f aca="false">Y10*Вводные!$B$19</f>
+      <c r="Y12" s="15" t="n">
+        <f aca="false">Y10*Вводные!$B$22</f>
         <v>327.3</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="22" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B13" s="23" t="n">
-        <f aca="false">B9-B11-B12</f>
-        <v>18565.6</v>
+        <f aca="false">B9-B11-B12-B4*Вводные!$B$12</f>
+        <v>43726.24</v>
       </c>
       <c r="C13" s="23" t="n">
-        <f aca="false">C9-C11-C12</f>
-        <v>20030.848</v>
+        <f aca="false">C9-C11-C12-C4*Вводные!$B$12</f>
+        <v>47204.3392</v>
       </c>
       <c r="D13" s="23" t="n">
-        <f aca="false">D9-D11-D12</f>
-        <v>25304.444</v>
+        <f aca="false">D9-D11-D12-D4*Вводные!$B$12</f>
+        <v>59936.7176</v>
       </c>
       <c r="E13" s="23" t="n">
-        <f aca="false">E9-E11-E12</f>
-        <v>27362.2456</v>
+        <f aca="false">E9-E11-E12-E4*Вводные!$B$12</f>
+        <v>64810.39024</v>
       </c>
       <c r="F13" s="23" t="n">
-        <f aca="false">F9-F11-F12</f>
-        <v>29531.1608</v>
+        <f aca="false">F9-F11-F12-F4*Вводные!$B$12</f>
+        <v>69947.58032</v>
       </c>
       <c r="G13" s="23" t="n">
-        <f aca="false">G9-G11-G12</f>
-        <v>31922.6032</v>
+        <f aca="false">G9-G11-G12-G4*Вводные!$B$12</f>
+        <v>75612.10528</v>
       </c>
       <c r="H13" s="23" t="n">
-        <f aca="false">H9-H11-H12</f>
-        <v>34517.9872</v>
+        <f aca="false">H9-H11-H12-H4*Вводные!$B$12</f>
+        <v>81758.77888</v>
       </c>
       <c r="I13" s="23" t="n">
-        <f aca="false">I9-I11-I12</f>
-        <v>37242.9704</v>
+        <f aca="false">I9-I11-I12-I4*Вводные!$B$12</f>
+        <v>88214.05616</v>
       </c>
       <c r="J13" s="23" t="n">
-        <f aca="false">J9-J11-J12</f>
-        <v>40190.4808</v>
+        <f aca="false">J9-J11-J12-J4*Вводные!$B$12</f>
+        <v>95196.66832</v>
       </c>
       <c r="K13" s="23" t="n">
-        <f aca="false">K9-K11-K12</f>
-        <v>43434.7608</v>
+        <f aca="false">K9-K11-K12-K4*Вводные!$B$12</f>
+        <v>102880.06032</v>
       </c>
       <c r="L13" s="23" t="n">
-        <f aca="false">L9-L11-L12</f>
-        <v>46901.368</v>
+        <f aca="false">L9-L11-L12-L4*Вводные!$B$12</f>
+        <v>111090.5872</v>
       </c>
       <c r="M13" s="23" t="n">
-        <f aca="false">M9-M11-M12</f>
-        <v>50701.716</v>
+        <f aca="false">M9-M11-M12-M4*Вводные!$B$12</f>
+        <v>120092.0664</v>
       </c>
       <c r="N13" s="23" t="n">
-        <f aca="false">N9-N11-N12</f>
-        <v>54724.3912</v>
+        <f aca="false">N9-N11-N12-N4*Вводные!$B$12</f>
+        <v>129620.68048</v>
       </c>
       <c r="O13" s="23" t="n">
-        <f aca="false">O9-O11-O12</f>
-        <v>59080.8072</v>
+        <f aca="false">O9-O11-O12-O4*Вводные!$B$12</f>
+        <v>139940.24688</v>
       </c>
       <c r="P13" s="23" t="n">
-        <f aca="false">P9-P11-P12</f>
-        <v>63845.2064</v>
+        <f aca="false">P9-P11-P12-P4*Вводные!$B$12</f>
+        <v>151224.21056</v>
       </c>
       <c r="Q13" s="23" t="n">
-        <f aca="false">Q9-Q11-Q12</f>
-        <v>68943.1464</v>
+        <f aca="false">Q9-Q11-Q12-Q4*Вводные!$B$12</f>
+        <v>163298.92656</v>
       </c>
       <c r="R13" s="23" t="n">
-        <f aca="false">R9-R11-R12</f>
-        <v>74486.0408</v>
+        <f aca="false">R9-R11-R12-R4*Вводные!$B$12</f>
+        <v>176428.21232</v>
       </c>
       <c r="S13" s="23" t="n">
-        <f aca="false">S9-S11-S12</f>
-        <v>80455.304</v>
+        <f aca="false">S9-S11-S12-S4*Вводные!$B$12</f>
+        <v>190566.8816</v>
       </c>
       <c r="T13" s="23" t="n">
-        <f aca="false">T9-T11-T12</f>
-        <v>86869.4216</v>
+        <f aca="false">T9-T11-T12-T4*Вводные!$B$12</f>
+        <v>205760.02064</v>
       </c>
       <c r="U13" s="23" t="n">
-        <f aca="false">U9-U11-U12</f>
-        <v>93821.2216</v>
+        <f aca="false">U9-U11-U12-U4*Вводные!$B$12</f>
+        <v>222226.26064</v>
       </c>
       <c r="V13" s="23" t="n">
-        <f aca="false">V9-V11-V12</f>
-        <v>101310.604</v>
+        <f aca="false">V9-V11-V12-V4*Вводные!$B$12</f>
+        <v>239965.5016</v>
       </c>
       <c r="W13" s="23" t="n">
-        <f aca="false">W9-W11-W12</f>
-        <v>109448.8824</v>
+        <f aca="false">W9-W11-W12-W4*Вводные!$B$12</f>
+        <v>259241.46096</v>
       </c>
       <c r="X13" s="23" t="n">
-        <f aca="false">X9-X11-X12</f>
-        <v>118235.9568</v>
+        <f aca="false">X9-X11-X12-X4*Вводные!$B$12</f>
+        <v>280054.03872</v>
       </c>
       <c r="Y13" s="23" t="n">
-        <f aca="false">Y9-Y11-Y12</f>
-        <v>127690.3128</v>
+        <f aca="false">Y9-Y11-Y12-Y4*Вводные!$B$12</f>
+        <v>302448.32112</v>
       </c>
       <c r="Z13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="B14" s="13" t="n">
-        <f aca="false">IF(1&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+        <v>97</v>
+      </c>
+      <c r="B14" s="15" t="n">
+        <f aca="false">IF(1&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="C14" s="13" t="n">
-        <f aca="false">IF(2&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="C14" s="15" t="n">
+        <f aca="false">IF(2&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="D14" s="13" t="n">
-        <f aca="false">IF(3&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="D14" s="15" t="n">
+        <f aca="false">IF(3&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="E14" s="13" t="n">
-        <f aca="false">IF(4&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="E14" s="15" t="n">
+        <f aca="false">IF(4&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="F14" s="13" t="n">
-        <f aca="false">IF(5&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="F14" s="15" t="n">
+        <f aca="false">IF(5&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="G14" s="13" t="n">
-        <f aca="false">IF(6&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="G14" s="15" t="n">
+        <f aca="false">IF(6&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="H14" s="13" t="n">
-        <f aca="false">IF(7&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="H14" s="15" t="n">
+        <f aca="false">IF(7&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="I14" s="13" t="n">
-        <f aca="false">IF(8&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="I14" s="15" t="n">
+        <f aca="false">IF(8&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="J14" s="13" t="n">
-        <f aca="false">IF(9&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="J14" s="15" t="n">
+        <f aca="false">IF(9&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="K14" s="13" t="n">
-        <f aca="false">IF(10&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="K14" s="15" t="n">
+        <f aca="false">IF(10&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="L14" s="13" t="n">
-        <f aca="false">IF(11&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="L14" s="15" t="n">
+        <f aca="false">IF(11&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="M14" s="13" t="n">
-        <f aca="false">IF(12&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="M14" s="15" t="n">
+        <f aca="false">IF(12&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>8000</v>
       </c>
-      <c r="N14" s="13" t="n">
-        <f aca="false">IF(13&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="N14" s="15" t="n">
+        <f aca="false">IF(13&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="O14" s="13" t="n">
-        <f aca="false">IF(14&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="O14" s="15" t="n">
+        <f aca="false">IF(14&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="P14" s="13" t="n">
-        <f aca="false">IF(15&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="P14" s="15" t="n">
+        <f aca="false">IF(15&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="Q14" s="13" t="n">
-        <f aca="false">IF(16&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="Q14" s="15" t="n">
+        <f aca="false">IF(16&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="R14" s="13" t="n">
-        <f aca="false">IF(17&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="R14" s="15" t="n">
+        <f aca="false">IF(17&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="S14" s="13" t="n">
-        <f aca="false">IF(18&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="S14" s="15" t="n">
+        <f aca="false">IF(18&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="T14" s="13" t="n">
-        <f aca="false">IF(19&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="T14" s="15" t="n">
+        <f aca="false">IF(19&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="U14" s="13" t="n">
-        <f aca="false">IF(20&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="U14" s="15" t="n">
+        <f aca="false">IF(20&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="V14" s="13" t="n">
-        <f aca="false">IF(21&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="V14" s="15" t="n">
+        <f aca="false">IF(21&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="W14" s="13" t="n">
-        <f aca="false">IF(22&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="W14" s="15" t="n">
+        <f aca="false">IF(22&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="X14" s="13" t="n">
-        <f aca="false">IF(23&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="X14" s="15" t="n">
+        <f aca="false">IF(23&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
-      <c r="Y14" s="13" t="n">
-        <f aca="false">IF(24&gt;12,Вводные!$B$21*Вводные!$B$22,Вводные!$B$21)</f>
+      <c r="Y14" s="15" t="n">
+        <f aca="false">IF(24&gt;12,Вводные!$B$24*Вводные!$B$25,Вводные!$B$24)</f>
         <v>12000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="B15" s="13" t="n">
-        <f aca="false">B9*Вводные!$B$23</f>
-        <v>2880</v>
-      </c>
-      <c r="C15" s="13" t="n">
-        <f aca="false">C9*Вводные!$B$23</f>
-        <v>3110.4</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <f aca="false">D9*Вводные!$B$23</f>
-        <v>3931.2</v>
-      </c>
-      <c r="E15" s="13" t="n">
-        <f aca="false">E9*Вводные!$B$23</f>
-        <v>4250.88</v>
-      </c>
-      <c r="F15" s="13" t="n">
-        <f aca="false">F9*Вводные!$B$23</f>
-        <v>4587.84</v>
-      </c>
-      <c r="G15" s="13" t="n">
-        <f aca="false">G9*Вводные!$B$23</f>
-        <v>4959.36</v>
-      </c>
-      <c r="H15" s="13" t="n">
-        <f aca="false">H9*Вводные!$B$23</f>
-        <v>5362.56</v>
-      </c>
-      <c r="I15" s="13" t="n">
-        <f aca="false">I9*Вводные!$B$23</f>
-        <v>5785.92</v>
-      </c>
-      <c r="J15" s="13" t="n">
-        <f aca="false">J9*Вводные!$B$23</f>
-        <v>6243.84</v>
-      </c>
-      <c r="K15" s="13" t="n">
-        <f aca="false">K9*Вводные!$B$23</f>
-        <v>6747.84</v>
-      </c>
-      <c r="L15" s="13" t="n">
-        <f aca="false">L9*Вводные!$B$23</f>
-        <v>7286.4</v>
-      </c>
-      <c r="M15" s="13" t="n">
-        <f aca="false">M9*Вводные!$B$23</f>
-        <v>7876.8</v>
-      </c>
-      <c r="N15" s="13" t="n">
-        <f aca="false">N9*Вводные!$B$23</f>
-        <v>8501.76</v>
-      </c>
-      <c r="O15" s="13" t="n">
-        <f aca="false">O9*Вводные!$B$23</f>
-        <v>9178.56</v>
-      </c>
-      <c r="P15" s="13" t="n">
-        <f aca="false">P9*Вводные!$B$23</f>
-        <v>9918.72</v>
-      </c>
-      <c r="Q15" s="13" t="n">
-        <f aca="false">Q9*Вводные!$B$23</f>
-        <v>10710.72</v>
-      </c>
-      <c r="R15" s="13" t="n">
-        <f aca="false">R9*Вводные!$B$23</f>
-        <v>11571.84</v>
-      </c>
-      <c r="S15" s="13" t="n">
-        <f aca="false">S9*Вводные!$B$23</f>
-        <v>12499.2</v>
-      </c>
-      <c r="T15" s="13" t="n">
-        <f aca="false">T9*Вводные!$B$23</f>
-        <v>13495.68</v>
-      </c>
-      <c r="U15" s="13" t="n">
-        <f aca="false">U9*Вводные!$B$23</f>
-        <v>14575.68</v>
-      </c>
-      <c r="V15" s="13" t="n">
-        <f aca="false">V9*Вводные!$B$23</f>
-        <v>15739.2</v>
-      </c>
-      <c r="W15" s="13" t="n">
-        <f aca="false">W9*Вводные!$B$23</f>
-        <v>17003.52</v>
-      </c>
-      <c r="X15" s="13" t="n">
-        <f aca="false">X9*Вводные!$B$23</f>
-        <v>18368.64</v>
-      </c>
-      <c r="Y15" s="13" t="n">
-        <f aca="false">Y9*Вводные!$B$23</f>
-        <v>19837.44</v>
+        <v>98</v>
+      </c>
+      <c r="B15" s="15" t="n">
+        <f aca="false">B9*Вводные!$B$26</f>
+        <v>7002</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <f aca="false">C9*Вводные!$B$26</f>
+        <v>7562.16</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <f aca="false">D9*Вводные!$B$26</f>
+        <v>9557.73</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <f aca="false">E9*Вводные!$B$26</f>
+        <v>10334.952</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <f aca="false">F9*Вводные!$B$26</f>
+        <v>11154.186</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <f aca="false">G9*Вводные!$B$26</f>
+        <v>12057.444</v>
+      </c>
+      <c r="H15" s="15" t="n">
+        <f aca="false">H9*Вводные!$B$26</f>
+        <v>13037.724</v>
+      </c>
+      <c r="I15" s="15" t="n">
+        <f aca="false">I9*Вводные!$B$26</f>
+        <v>14067.018</v>
+      </c>
+      <c r="J15" s="15" t="n">
+        <f aca="false">J9*Вводные!$B$26</f>
+        <v>15180.336</v>
+      </c>
+      <c r="K15" s="15" t="n">
+        <f aca="false">K9*Вводные!$B$26</f>
+        <v>16405.686</v>
+      </c>
+      <c r="L15" s="15" t="n">
+        <f aca="false">L9*Вводные!$B$26</f>
+        <v>17715.06</v>
+      </c>
+      <c r="M15" s="15" t="n">
+        <f aca="false">M9*Вводные!$B$26</f>
+        <v>19150.47</v>
+      </c>
+      <c r="N15" s="15" t="n">
+        <f aca="false">N9*Вводные!$B$26</f>
+        <v>20669.904</v>
+      </c>
+      <c r="O15" s="15" t="n">
+        <f aca="false">O9*Вводные!$B$26</f>
+        <v>22315.374</v>
+      </c>
+      <c r="P15" s="15" t="n">
+        <f aca="false">P9*Вводные!$B$26</f>
+        <v>24114.888</v>
+      </c>
+      <c r="Q15" s="15" t="n">
+        <f aca="false">Q9*Вводные!$B$26</f>
+        <v>26040.438</v>
+      </c>
+      <c r="R15" s="15" t="n">
+        <f aca="false">R9*Вводные!$B$26</f>
+        <v>28134.036</v>
+      </c>
+      <c r="S15" s="15" t="n">
+        <f aca="false">S9*Вводные!$B$26</f>
+        <v>30388.68</v>
+      </c>
+      <c r="T15" s="15" t="n">
+        <f aca="false">T9*Вводные!$B$26</f>
+        <v>32811.372</v>
+      </c>
+      <c r="U15" s="15" t="n">
+        <f aca="false">U9*Вводные!$B$26</f>
+        <v>35437.122</v>
+      </c>
+      <c r="V15" s="15" t="n">
+        <f aca="false">V9*Вводные!$B$26</f>
+        <v>38265.93</v>
+      </c>
+      <c r="W15" s="15" t="n">
+        <f aca="false">W9*Вводные!$B$26</f>
+        <v>41339.808</v>
+      </c>
+      <c r="X15" s="15" t="n">
+        <f aca="false">X9*Вводные!$B$26</f>
+        <v>44658.756</v>
+      </c>
+      <c r="Y15" s="15" t="n">
+        <f aca="false">Y9*Вводные!$B$26</f>
+        <v>48229.776</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="B16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+        <v>99</v>
+      </c>
+      <c r="B16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="C16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="C16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="D16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="D16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="E16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="E16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="F16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="F16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="G16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="G16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="H16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="H16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="I16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="I16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="J16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="J16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="K16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="K16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="L16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="L16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="M16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="M16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="N16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="N16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="O16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="O16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="P16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="P16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="Q16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="Q16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="R16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="R16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="S16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="S16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="T16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="T16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="U16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="U16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="V16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="V16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="W16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="W16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="X16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="X16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
-      <c r="Y16" s="13" t="n">
-        <f aca="false">Вводные!$B$20+Вводные!$B$24</f>
+      <c r="Y16" s="15" t="n">
+        <f aca="false">Вводные!$B$23+Вводные!$B$27</f>
         <v>630</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B17" s="23" t="n">
         <f aca="false">B13-B14-B15-B16</f>
-        <v>7055.6</v>
+        <v>28094.24</v>
       </c>
       <c r="C17" s="23" t="n">
         <f aca="false">C13-C14-C15-C16</f>
-        <v>8290.448</v>
+        <v>31012.1792</v>
       </c>
       <c r="D17" s="23" t="n">
         <f aca="false">D13-D14-D15-D16</f>
-        <v>12743.244</v>
+        <v>41748.9876</v>
       </c>
       <c r="E17" s="23" t="n">
         <f aca="false">E13-E14-E15-E16</f>
-        <v>14481.3656</v>
+        <v>45845.43824</v>
       </c>
       <c r="F17" s="23" t="n">
         <f aca="false">F13-F14-F15-F16</f>
-        <v>16313.3208</v>
+        <v>50163.39432</v>
       </c>
       <c r="G17" s="23" t="n">
         <f aca="false">G13-G14-G15-G16</f>
-        <v>18333.2432</v>
+        <v>54924.66128</v>
       </c>
       <c r="H17" s="23" t="n">
         <f aca="false">H13-H14-H15-H16</f>
-        <v>20525.4272</v>
+        <v>60091.05488</v>
       </c>
       <c r="I17" s="23" t="n">
         <f aca="false">I13-I14-I15-I16</f>
-        <v>22827.0504</v>
+        <v>65517.03816</v>
       </c>
       <c r="J17" s="23" t="n">
         <f aca="false">J13-J14-J15-J16</f>
-        <v>25316.6408</v>
+        <v>71386.33232</v>
       </c>
       <c r="K17" s="23" t="n">
         <f aca="false">K13-K14-K15-K16</f>
-        <v>28056.9208</v>
+        <v>77844.37432</v>
       </c>
       <c r="L17" s="23" t="n">
         <f aca="false">L13-L14-L15-L16</f>
-        <v>30984.968</v>
+        <v>84745.5272</v>
       </c>
       <c r="M17" s="23" t="n">
         <f aca="false">M13-M14-M15-M16</f>
-        <v>34194.916</v>
+        <v>92311.5964</v>
       </c>
       <c r="N17" s="23" t="n">
         <f aca="false">N13-N14-N15-N16</f>
-        <v>33592.6312</v>
+        <v>96320.77648</v>
       </c>
       <c r="O17" s="23" t="n">
         <f aca="false">O13-O14-O15-O16</f>
-        <v>37272.2472</v>
+        <v>104994.87288</v>
       </c>
       <c r="P17" s="23" t="n">
         <f aca="false">P13-P14-P15-P16</f>
-        <v>41296.4864</v>
+        <v>114479.32256</v>
       </c>
       <c r="Q17" s="23" t="n">
         <f aca="false">Q13-Q14-Q15-Q16</f>
-        <v>45602.4264</v>
+        <v>124628.48856</v>
       </c>
       <c r="R17" s="23" t="n">
         <f aca="false">R13-R14-R15-R16</f>
-        <v>50284.2008</v>
+        <v>135664.17632</v>
       </c>
       <c r="S17" s="23" t="n">
         <f aca="false">S13-S14-S15-S16</f>
-        <v>55326.104</v>
+        <v>147548.2016</v>
       </c>
       <c r="T17" s="23" t="n">
         <f aca="false">T13-T14-T15-T16</f>
-        <v>60743.7416</v>
+        <v>160318.64864</v>
       </c>
       <c r="U17" s="23" t="n">
         <f aca="false">U13-U14-U15-U16</f>
-        <v>66615.5416</v>
+        <v>174159.13864</v>
       </c>
       <c r="V17" s="23" t="n">
         <f aca="false">V13-V14-V15-V16</f>
-        <v>72941.404</v>
+        <v>189069.5716</v>
       </c>
       <c r="W17" s="23" t="n">
         <f aca="false">W13-W14-W15-W16</f>
-        <v>79815.3624</v>
+        <v>205271.65296</v>
       </c>
       <c r="X17" s="23" t="n">
         <f aca="false">X13-X14-X15-X16</f>
-        <v>87237.3168</v>
+        <v>222765.28272</v>
       </c>
       <c r="Y17" s="23" t="n">
         <f aca="false">Y13-Y14-Y15-Y16</f>
-        <v>95222.8728</v>
+        <v>241588.54512</v>
       </c>
       <c r="Z17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="B18" s="23" t="n">
-        <f aca="false">Вводные!$B$27+B17</f>
-        <v>157055.6</v>
+        <f aca="false">Вводные!$B$30+B17</f>
+        <v>178094.24</v>
       </c>
       <c r="C18" s="23" t="n">
         <f aca="false">B18+C17</f>
-        <v>165346.048</v>
+        <v>209106.4192</v>
       </c>
       <c r="D18" s="23" t="n">
         <f aca="false">C18+D17</f>
-        <v>178089.292</v>
+        <v>250855.4068</v>
       </c>
       <c r="E18" s="23" t="n">
         <f aca="false">D18+E17</f>
-        <v>192570.6576</v>
+        <v>296700.84504</v>
       </c>
       <c r="F18" s="23" t="n">
         <f aca="false">E18+F17</f>
-        <v>208883.9784</v>
+        <v>346864.23936</v>
       </c>
       <c r="G18" s="23" t="n">
         <f aca="false">F18+G17</f>
-        <v>227217.2216</v>
+        <v>401788.90064</v>
       </c>
       <c r="H18" s="23" t="n">
         <f aca="false">G18+H17</f>
-        <v>247742.6488</v>
+        <v>461879.95552</v>
       </c>
       <c r="I18" s="23" t="n">
         <f aca="false">H18+I17</f>
-        <v>270569.6992</v>
+        <v>527396.99368</v>
       </c>
       <c r="J18" s="23" t="n">
         <f aca="false">I18+J17</f>
-        <v>295886.34</v>
+        <v>598783.326</v>
       </c>
       <c r="K18" s="23" t="n">
         <f aca="false">J18+K17</f>
-        <v>323943.2608</v>
+        <v>676627.70032</v>
       </c>
       <c r="L18" s="23" t="n">
         <f aca="false">K18+L17</f>
-        <v>354928.2288</v>
+        <v>761373.22752</v>
       </c>
       <c r="M18" s="23" t="n">
         <f aca="false">L18+M17</f>
-        <v>389123.1448</v>
+        <v>853684.82392</v>
       </c>
       <c r="N18" s="23" t="n">
         <f aca="false">M18+N17</f>
-        <v>422715.776</v>
+        <v>950005.6004</v>
       </c>
       <c r="O18" s="23" t="n">
         <f aca="false">N18+O17</f>
-        <v>459988.0232</v>
+        <v>1055000.47328</v>
       </c>
       <c r="P18" s="23" t="n">
         <f aca="false">O18+P17</f>
-        <v>501284.5096</v>
+        <v>1169479.79584</v>
       </c>
       <c r="Q18" s="23" t="n">
         <f aca="false">P18+Q17</f>
-        <v>546886.936</v>
+        <v>1294108.2844</v>
       </c>
       <c r="R18" s="23" t="n">
         <f aca="false">Q18+R17</f>
-        <v>597171.1368</v>
+        <v>1429772.46072</v>
       </c>
       <c r="S18" s="23" t="n">
         <f aca="false">R18+S17</f>
-        <v>652497.2408</v>
+        <v>1577320.66232</v>
       </c>
       <c r="T18" s="23" t="n">
         <f aca="false">S18+T17</f>
-        <v>713240.9824</v>
+        <v>1737639.31096</v>
       </c>
       <c r="U18" s="23" t="n">
         <f aca="false">T18+U17</f>
-        <v>779856.524</v>
+        <v>1911798.4496</v>
       </c>
       <c r="V18" s="23" t="n">
         <f aca="false">U18+V17</f>
-        <v>852797.928</v>
+        <v>2100868.0212</v>
       </c>
       <c r="W18" s="23" t="n">
         <f aca="false">V18+W17</f>
-        <v>932613.2904</v>
+        <v>2306139.67416</v>
       </c>
       <c r="X18" s="23" t="n">
         <f aca="false">W18+X17</f>
-        <v>1019850.6072</v>
+        <v>2528904.95688</v>
       </c>
       <c r="Y18" s="23" t="n">
         <f aca="false">X18+Y17</f>
-        <v>1115073.48</v>
+        <v>2770493.502</v>
       </c>
       <c r="Z18" s="24"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="25" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -3018,88 +3080,88 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B3" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!B9:M9)</f>
-        <v>420153.6</v>
+        <v>1021498.44</v>
       </c>
       <c r="C3" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!N9:Y9)</f>
-        <v>1076006.4</v>
+        <v>2616040.56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B4" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!B13:M13)</f>
-        <v>405706.1848</v>
+        <v>960469.58992</v>
       </c>
       <c r="C4" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!N13:Y13)</f>
-        <v>1038911.2952</v>
+        <v>2460774.76208</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B5" s="27" t="n">
         <f aca="false">B4/B3</f>
-        <v>0.965613967844141</v>
+        <v>0.940255562132821</v>
       </c>
       <c r="C5" s="27" t="n">
         <f aca="false">C4/C3</f>
-        <v>0.965525200593602</v>
+        <v>0.94064855098424</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B6" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!B17:M17)</f>
-        <v>239123.1448</v>
+        <v>703684.82392</v>
       </c>
       <c r="C6" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!N17:Y17)</f>
-        <v>725950.3352</v>
+        <v>1916808.67808</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B6/B3</f>
-        <v>0.569132681000472</v>
+        <v>0.688875084253677</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C6/C3</f>
-        <v>0.674671019800626</v>
+        <v>0.732713669424147</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B8" s="28" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!B3:M3)</f>
@@ -3112,74 +3174,74 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B9" s="26" t="n">
         <f aca="false">'Прогноз 24 мес'!M18</f>
-        <v>389123.1448</v>
+        <v>853684.82392</v>
       </c>
       <c r="C9" s="26" t="n">
         <f aca="false">'Прогноз 24 мес'!Y18</f>
-        <v>1115073.48</v>
+        <v>2770493.502</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="29" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="13" t="n">
-        <f aca="false">Вводные!B11</f>
-        <v>960</v>
+        <v>113</v>
+      </c>
+      <c r="B12" s="15" t="n">
+        <f aca="false">Вводные!B14</f>
+        <v>2334</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="B13" s="13" t="n">
-        <f aca="false">Вводные!B11*(1+Вводные!B12)</f>
-        <v>1152</v>
+        <v>114</v>
+      </c>
+      <c r="B13" s="15" t="n">
+        <f aca="false">Вводные!B14*(1+Вводные!B15)</f>
+        <v>2800.8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="B14" s="13" t="n">
-        <f aca="false">Вводные!B28</f>
+        <v>115</v>
+      </c>
+      <c r="B14" s="15" t="n">
+        <f aca="false">Вводные!B31</f>
         <v>60</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B15" s="30" t="n">
         <f aca="false">B13/B14</f>
-        <v>19.2</v>
+        <v>46.68</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="B16" s="13" t="n">
-        <f aca="false">Вводные!B11*Вводные!B18+Вводные!B19*3</f>
-        <v>33.72</v>
+        <v>117</v>
+      </c>
+      <c r="B16" s="15" t="n">
+        <f aca="false">Вводные!B14*Вводные!B21+Вводные!B22*3+(1-Вводные!B13)*Вводные!B12</f>
+        <v>149.688</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="B17" s="13" t="n">
+        <v>118</v>
+      </c>
+      <c r="B17" s="15" t="n">
         <f aca="false">B12-B16</f>
-        <v>926.28</v>
+        <v>2184.312</v>
       </c>
     </row>
   </sheetData>
@@ -3207,41 +3269,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="B3" s="12" t="n">
+        <v>123</v>
+      </c>
+      <c r="B3" s="14" t="n">
         <v>0.04</v>
       </c>
       <c r="C3" s="27" t="n">
-        <f aca="false">Вводные!B15</f>
+        <f aca="false">Вводные!B18</f>
         <v>0.08</v>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="14" t="n">
         <v>0.12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">Вводные!$B$5*(((1+B3)^24)-1)/B3</f>
@@ -3258,41 +3320,41 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="B5" s="13" t="n">
-        <f aca="false">B4*Вводные!$B$11*(1+Вводные!$B$12)</f>
-        <v>900463.198977649</v>
-      </c>
-      <c r="C5" s="13" t="n">
-        <f aca="false">C4*Вводные!$B$11*(1+Вводные!$B$12)</f>
-        <v>1538260.05232515</v>
-      </c>
-      <c r="D5" s="13" t="n">
-        <f aca="false">D4*Вводные!$B$11*(1+Вводные!$B$12)</f>
-        <v>2722296.75542447</v>
+        <v>125</v>
+      </c>
+      <c r="B5" s="15" t="n">
+        <f aca="false">B4*Вводные!$B$14*(1+Вводные!$B$15)</f>
+        <v>2189251.15251441</v>
+      </c>
+      <c r="C5" s="15" t="n">
+        <f aca="false">C4*Вводные!$B$14*(1+Вводные!$B$15)</f>
+        <v>3739894.75221553</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <f aca="false">D4*Вводные!$B$14*(1+Вводные!$B$15)</f>
+        <v>6618583.98662574</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="B6" s="13" t="n">
-        <f aca="false">Вводные!$B$5*((1+B3)^23)*Вводные!$B$11*(1+Вводные!$B$12)</f>
-        <v>56787.046114525</v>
-      </c>
-      <c r="C6" s="13" t="n">
-        <f aca="false">Вводные!$B$5*((1+C3)^23)*Вводные!$B$11*(1+Вводные!$B$12)</f>
-        <v>135278.522394456</v>
-      </c>
-      <c r="D6" s="13" t="n">
-        <f aca="false">Вводные!$B$5*((1+D3)^23)*Вводные!$B$11*(1+Вводные!$B$12)</f>
-        <v>312246.080938336</v>
+        <v>126</v>
+      </c>
+      <c r="B6" s="15" t="n">
+        <f aca="false">Вводные!$B$5*((1+B3)^23)*Вводные!$B$14*(1+Вводные!$B$15)</f>
+        <v>138063.505865939</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <f aca="false">Вводные!$B$5*((1+C3)^23)*Вводные!$B$14*(1+Вводные!$B$15)</f>
+        <v>328895.907571521</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <f aca="false">Вводные!$B$5*((1+D3)^23)*Вводные!$B$14*(1+Вводные!$B$15)</f>
+        <v>759148.284281328</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="25" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clarify formula gift terms across plans
Karen sends his formula as a gift on BOTH support plans: on the 5-week
plan the client pays the $180 delivery, on the 100-day plan Karen
covers delivery himself; the $500 review does not include the formula.
Updated payment page descriptions (RU/EN), the post-payment page, the
assistant prompt, and the financial model (gift cost now applies to
every new client).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/launch/Финансовая_модель_Python_Method.xlsx
+++ b/docs/launch/Финансовая_модель_Python_Method.xlsx
@@ -116,7 +116,7 @@
     <t xml:space="preserve">Себестоимость формулы и доставки, $</t>
   </si>
   <si>
-    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — во сколько центру обходится формула + отправка. Замените фактом.</t>
+    <t xml:space="preserve">ПРЕДПОЛОЖЕНИЕ — себестоимость формулы + отправки. Подарок идёт на ОБОИХ тарифах (на «100 дней» доставка за счёт центра). Замените фактом.</t>
   </si>
   <si>
     <t xml:space="preserve">Доля клиентов, выбирающих «100 дней»</t>
@@ -1148,7 +1148,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
         <v>29</v>
       </c>
@@ -2446,100 +2446,100 @@
         <v>96</v>
       </c>
       <c r="B13" s="23" t="n">
-        <f aca="false">B9-B11-B12-B4*Вводные!$B$12</f>
-        <v>43726.24</v>
+        <f aca="false">B9-B11-B12-B3*Вводные!$B$12</f>
+        <v>42766.24</v>
       </c>
       <c r="C13" s="23" t="n">
-        <f aca="false">C9-C11-C12-C4*Вводные!$B$12</f>
-        <v>47204.3392</v>
+        <f aca="false">C9-C11-C12-C3*Вводные!$B$12</f>
+        <v>46167.5392</v>
       </c>
       <c r="D13" s="23" t="n">
-        <f aca="false">D9-D11-D12-D4*Вводные!$B$12</f>
-        <v>59936.7176</v>
+        <f aca="false">D9-D11-D12-D3*Вводные!$B$12</f>
+        <v>58818.3176</v>
       </c>
       <c r="E13" s="23" t="n">
-        <f aca="false">E9-E11-E12-E4*Вводные!$B$12</f>
-        <v>64810.39024</v>
+        <f aca="false">E9-E11-E12-E3*Вводные!$B$12</f>
+        <v>63600.79024</v>
       </c>
       <c r="F13" s="23" t="n">
-        <f aca="false">F9-F11-F12-F4*Вводные!$B$12</f>
-        <v>69947.58032</v>
+        <f aca="false">F9-F11-F12-F3*Вводные!$B$12</f>
+        <v>68641.98032</v>
       </c>
       <c r="G13" s="23" t="n">
-        <f aca="false">G9-G11-G12-G4*Вводные!$B$12</f>
-        <v>75612.10528</v>
+        <f aca="false">G9-G11-G12-G3*Вводные!$B$12</f>
+        <v>74200.90528</v>
       </c>
       <c r="H13" s="23" t="n">
-        <f aca="false">H9-H11-H12-H4*Вводные!$B$12</f>
-        <v>81758.77888</v>
+        <f aca="false">H9-H11-H12-H3*Вводные!$B$12</f>
+        <v>80232.37888</v>
       </c>
       <c r="I13" s="23" t="n">
-        <f aca="false">I9-I11-I12-I4*Вводные!$B$12</f>
-        <v>88214.05616</v>
+        <f aca="false">I9-I11-I12-I3*Вводные!$B$12</f>
+        <v>86567.65616</v>
       </c>
       <c r="J13" s="23" t="n">
-        <f aca="false">J9-J11-J12-J4*Вводные!$B$12</f>
-        <v>95196.66832</v>
+        <f aca="false">J9-J11-J12-J3*Вводные!$B$12</f>
+        <v>93420.66832</v>
       </c>
       <c r="K13" s="23" t="n">
-        <f aca="false">K9-K11-K12-K4*Вводные!$B$12</f>
-        <v>102880.06032</v>
+        <f aca="false">K9-K11-K12-K3*Вводные!$B$12</f>
+        <v>100960.06032</v>
       </c>
       <c r="L13" s="23" t="n">
-        <f aca="false">L9-L11-L12-L4*Вводные!$B$12</f>
-        <v>111090.5872</v>
+        <f aca="false">L9-L11-L12-L3*Вводные!$B$12</f>
+        <v>109016.9872</v>
       </c>
       <c r="M13" s="23" t="n">
-        <f aca="false">M9-M11-M12-M4*Вводные!$B$12</f>
-        <v>120092.0664</v>
+        <f aca="false">M9-M11-M12-M3*Вводные!$B$12</f>
+        <v>117850.4664</v>
       </c>
       <c r="N13" s="23" t="n">
-        <f aca="false">N9-N11-N12-N4*Вводные!$B$12</f>
-        <v>129620.68048</v>
+        <f aca="false">N9-N11-N12-N3*Вводные!$B$12</f>
+        <v>127201.48048</v>
       </c>
       <c r="O13" s="23" t="n">
-        <f aca="false">O9-O11-O12-O4*Вводные!$B$12</f>
-        <v>139940.24688</v>
+        <f aca="false">O9-O11-O12-O3*Вводные!$B$12</f>
+        <v>137329.04688</v>
       </c>
       <c r="P13" s="23" t="n">
-        <f aca="false">P9-P11-P12-P4*Вводные!$B$12</f>
-        <v>151224.21056</v>
+        <f aca="false">P9-P11-P12-P3*Вводные!$B$12</f>
+        <v>148401.81056</v>
       </c>
       <c r="Q13" s="23" t="n">
-        <f aca="false">Q9-Q11-Q12-Q4*Вводные!$B$12</f>
-        <v>163298.92656</v>
+        <f aca="false">Q9-Q11-Q12-Q3*Вводные!$B$12</f>
+        <v>160250.92656</v>
       </c>
       <c r="R13" s="23" t="n">
-        <f aca="false">R9-R11-R12-R4*Вводные!$B$12</f>
-        <v>176428.21232</v>
+        <f aca="false">R9-R11-R12-R3*Вводные!$B$12</f>
+        <v>173135.41232</v>
       </c>
       <c r="S13" s="23" t="n">
-        <f aca="false">S9-S11-S12-S4*Вводные!$B$12</f>
-        <v>190566.8816</v>
+        <f aca="false">S9-S11-S12-S3*Вводные!$B$12</f>
+        <v>187010.0816</v>
       </c>
       <c r="T13" s="23" t="n">
-        <f aca="false">T9-T11-T12-T4*Вводные!$B$12</f>
-        <v>205760.02064</v>
+        <f aca="false">T9-T11-T12-T3*Вводные!$B$12</f>
+        <v>201920.02064</v>
       </c>
       <c r="U13" s="23" t="n">
-        <f aca="false">U9-U11-U12-U4*Вводные!$B$12</f>
-        <v>222226.26064</v>
+        <f aca="false">U9-U11-U12-U3*Вводные!$B$12</f>
+        <v>218079.06064</v>
       </c>
       <c r="V13" s="23" t="n">
-        <f aca="false">V9-V11-V12-V4*Вводные!$B$12</f>
-        <v>239965.5016</v>
+        <f aca="false">V9-V11-V12-V3*Вводные!$B$12</f>
+        <v>235487.1016</v>
       </c>
       <c r="W13" s="23" t="n">
-        <f aca="false">W9-W11-W12-W4*Вводные!$B$12</f>
-        <v>259241.46096</v>
+        <f aca="false">W9-W11-W12-W3*Вводные!$B$12</f>
+        <v>254403.06096</v>
       </c>
       <c r="X13" s="23" t="n">
-        <f aca="false">X9-X11-X12-X4*Вводные!$B$12</f>
-        <v>280054.03872</v>
+        <f aca="false">X9-X11-X12-X3*Вводные!$B$12</f>
+        <v>274826.83872</v>
       </c>
       <c r="Y13" s="23" t="n">
-        <f aca="false">Y9-Y11-Y12-Y4*Вводные!$B$12</f>
-        <v>302448.32112</v>
+        <f aca="false">Y9-Y11-Y12-Y3*Вводные!$B$12</f>
+        <v>296803.52112</v>
       </c>
       <c r="Z13" s="24"/>
     </row>
@@ -2852,99 +2852,99 @@
       </c>
       <c r="B17" s="23" t="n">
         <f aca="false">B13-B14-B15-B16</f>
-        <v>28094.24</v>
+        <v>27134.24</v>
       </c>
       <c r="C17" s="23" t="n">
         <f aca="false">C13-C14-C15-C16</f>
-        <v>31012.1792</v>
+        <v>29975.3792</v>
       </c>
       <c r="D17" s="23" t="n">
         <f aca="false">D13-D14-D15-D16</f>
-        <v>41748.9876</v>
+        <v>40630.5876</v>
       </c>
       <c r="E17" s="23" t="n">
         <f aca="false">E13-E14-E15-E16</f>
-        <v>45845.43824</v>
+        <v>44635.83824</v>
       </c>
       <c r="F17" s="23" t="n">
         <f aca="false">F13-F14-F15-F16</f>
-        <v>50163.39432</v>
+        <v>48857.79432</v>
       </c>
       <c r="G17" s="23" t="n">
         <f aca="false">G13-G14-G15-G16</f>
-        <v>54924.66128</v>
+        <v>53513.46128</v>
       </c>
       <c r="H17" s="23" t="n">
         <f aca="false">H13-H14-H15-H16</f>
-        <v>60091.05488</v>
+        <v>58564.65488</v>
       </c>
       <c r="I17" s="23" t="n">
         <f aca="false">I13-I14-I15-I16</f>
-        <v>65517.03816</v>
+        <v>63870.63816</v>
       </c>
       <c r="J17" s="23" t="n">
         <f aca="false">J13-J14-J15-J16</f>
-        <v>71386.33232</v>
+        <v>69610.33232</v>
       </c>
       <c r="K17" s="23" t="n">
         <f aca="false">K13-K14-K15-K16</f>
-        <v>77844.37432</v>
+        <v>75924.37432</v>
       </c>
       <c r="L17" s="23" t="n">
         <f aca="false">L13-L14-L15-L16</f>
-        <v>84745.5272</v>
+        <v>82671.9272</v>
       </c>
       <c r="M17" s="23" t="n">
         <f aca="false">M13-M14-M15-M16</f>
-        <v>92311.5964</v>
+        <v>90069.9964</v>
       </c>
       <c r="N17" s="23" t="n">
         <f aca="false">N13-N14-N15-N16</f>
-        <v>96320.77648</v>
+        <v>93901.57648</v>
       </c>
       <c r="O17" s="23" t="n">
         <f aca="false">O13-O14-O15-O16</f>
-        <v>104994.87288</v>
+        <v>102383.67288</v>
       </c>
       <c r="P17" s="23" t="n">
         <f aca="false">P13-P14-P15-P16</f>
-        <v>114479.32256</v>
+        <v>111656.92256</v>
       </c>
       <c r="Q17" s="23" t="n">
         <f aca="false">Q13-Q14-Q15-Q16</f>
-        <v>124628.48856</v>
+        <v>121580.48856</v>
       </c>
       <c r="R17" s="23" t="n">
         <f aca="false">R13-R14-R15-R16</f>
-        <v>135664.17632</v>
+        <v>132371.37632</v>
       </c>
       <c r="S17" s="23" t="n">
         <f aca="false">S13-S14-S15-S16</f>
-        <v>147548.2016</v>
+        <v>143991.4016</v>
       </c>
       <c r="T17" s="23" t="n">
         <f aca="false">T13-T14-T15-T16</f>
-        <v>160318.64864</v>
+        <v>156478.64864</v>
       </c>
       <c r="U17" s="23" t="n">
         <f aca="false">U13-U14-U15-U16</f>
-        <v>174159.13864</v>
+        <v>170011.93864</v>
       </c>
       <c r="V17" s="23" t="n">
         <f aca="false">V13-V14-V15-V16</f>
-        <v>189069.5716</v>
+        <v>184591.1716</v>
       </c>
       <c r="W17" s="23" t="n">
         <f aca="false">W13-W14-W15-W16</f>
-        <v>205271.65296</v>
+        <v>200433.25296</v>
       </c>
       <c r="X17" s="23" t="n">
         <f aca="false">X13-X14-X15-X16</f>
-        <v>222765.28272</v>
+        <v>217538.08272</v>
       </c>
       <c r="Y17" s="23" t="n">
         <f aca="false">Y13-Y14-Y15-Y16</f>
-        <v>241588.54512</v>
+        <v>235943.74512</v>
       </c>
       <c r="Z17" s="24"/>
     </row>
@@ -2954,99 +2954,99 @@
       </c>
       <c r="B18" s="23" t="n">
         <f aca="false">Вводные!$B$30+B17</f>
-        <v>178094.24</v>
+        <v>177134.24</v>
       </c>
       <c r="C18" s="23" t="n">
         <f aca="false">B18+C17</f>
-        <v>209106.4192</v>
+        <v>207109.6192</v>
       </c>
       <c r="D18" s="23" t="n">
         <f aca="false">C18+D17</f>
-        <v>250855.4068</v>
+        <v>247740.2068</v>
       </c>
       <c r="E18" s="23" t="n">
         <f aca="false">D18+E17</f>
-        <v>296700.84504</v>
+        <v>292376.04504</v>
       </c>
       <c r="F18" s="23" t="n">
         <f aca="false">E18+F17</f>
-        <v>346864.23936</v>
+        <v>341233.83936</v>
       </c>
       <c r="G18" s="23" t="n">
         <f aca="false">F18+G17</f>
-        <v>401788.90064</v>
+        <v>394747.30064</v>
       </c>
       <c r="H18" s="23" t="n">
         <f aca="false">G18+H17</f>
-        <v>461879.95552</v>
+        <v>453311.95552</v>
       </c>
       <c r="I18" s="23" t="n">
         <f aca="false">H18+I17</f>
-        <v>527396.99368</v>
+        <v>517182.59368</v>
       </c>
       <c r="J18" s="23" t="n">
         <f aca="false">I18+J17</f>
-        <v>598783.326</v>
+        <v>586792.926</v>
       </c>
       <c r="K18" s="23" t="n">
         <f aca="false">J18+K17</f>
-        <v>676627.70032</v>
+        <v>662717.30032</v>
       </c>
       <c r="L18" s="23" t="n">
         <f aca="false">K18+L17</f>
-        <v>761373.22752</v>
+        <v>745389.22752</v>
       </c>
       <c r="M18" s="23" t="n">
         <f aca="false">L18+M17</f>
-        <v>853684.82392</v>
+        <v>835459.22392</v>
       </c>
       <c r="N18" s="23" t="n">
         <f aca="false">M18+N17</f>
-        <v>950005.6004</v>
+        <v>929360.8004</v>
       </c>
       <c r="O18" s="23" t="n">
         <f aca="false">N18+O17</f>
-        <v>1055000.47328</v>
+        <v>1031744.47328</v>
       </c>
       <c r="P18" s="23" t="n">
         <f aca="false">O18+P17</f>
-        <v>1169479.79584</v>
+        <v>1143401.39584</v>
       </c>
       <c r="Q18" s="23" t="n">
         <f aca="false">P18+Q17</f>
-        <v>1294108.2844</v>
+        <v>1264981.8844</v>
       </c>
       <c r="R18" s="23" t="n">
         <f aca="false">Q18+R17</f>
-        <v>1429772.46072</v>
+        <v>1397353.26072</v>
       </c>
       <c r="S18" s="23" t="n">
         <f aca="false">R18+S17</f>
-        <v>1577320.66232</v>
+        <v>1541344.66232</v>
       </c>
       <c r="T18" s="23" t="n">
         <f aca="false">S18+T17</f>
-        <v>1737639.31096</v>
+        <v>1697823.31096</v>
       </c>
       <c r="U18" s="23" t="n">
         <f aca="false">T18+U17</f>
-        <v>1911798.4496</v>
+        <v>1867835.2496</v>
       </c>
       <c r="V18" s="23" t="n">
         <f aca="false">U18+V17</f>
-        <v>2100868.0212</v>
+        <v>2052426.4212</v>
       </c>
       <c r="W18" s="23" t="n">
         <f aca="false">V18+W17</f>
-        <v>2306139.67416</v>
+        <v>2252859.67416</v>
       </c>
       <c r="X18" s="23" t="n">
         <f aca="false">W18+X17</f>
-        <v>2528904.95688</v>
+        <v>2470397.75688</v>
       </c>
       <c r="Y18" s="23" t="n">
         <f aca="false">X18+Y17</f>
-        <v>2770493.502</v>
+        <v>2706341.502</v>
       </c>
       <c r="Z18" s="24"/>
     </row>
@@ -3113,11 +3113,11 @@
       </c>
       <c r="B4" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!B13:M13)</f>
-        <v>960469.58992</v>
+        <v>942243.98992</v>
       </c>
       <c r="C4" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!N13:Y13)</f>
-        <v>2460774.76208</v>
+        <v>2414848.36208</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3126,11 +3126,11 @@
       </c>
       <c r="B5" s="27" t="n">
         <f aca="false">B4/B3</f>
-        <v>0.940255562132821</v>
+        <v>0.922413537821947</v>
       </c>
       <c r="C5" s="27" t="n">
         <f aca="false">C4/C3</f>
-        <v>0.94064855098424</v>
+        <v>0.923092859875231</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3139,11 +3139,11 @@
       </c>
       <c r="B6" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!B17:M17)</f>
-        <v>703684.82392</v>
+        <v>685459.22392</v>
       </c>
       <c r="C6" s="26" t="n">
         <f aca="false">SUM('Прогноз 24 мес'!N17:Y17)</f>
-        <v>1916808.67808</v>
+        <v>1870882.27808</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3152,11 +3152,11 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B6/B3</f>
-        <v>0.688875084253677</v>
+        <v>0.671033059942803</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C6/C3</f>
-        <v>0.732713669424147</v>
+        <v>0.715157978315138</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3178,11 +3178,11 @@
       </c>
       <c r="B9" s="26" t="n">
         <f aca="false">'Прогноз 24 мес'!M18</f>
-        <v>853684.82392</v>
+        <v>835459.22392</v>
       </c>
       <c r="C9" s="26" t="n">
         <f aca="false">'Прогноз 24 мес'!Y18</f>
-        <v>2770493.502</v>
+        <v>2706341.502</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3231,8 +3231,8 @@
         <v>117</v>
       </c>
       <c r="B16" s="15" t="n">
-        <f aca="false">Вводные!B14*Вводные!B21+Вводные!B22*3+(1-Вводные!B13)*Вводные!B12</f>
-        <v>149.688</v>
+        <f aca="false">Вводные!B14*Вводные!B21+Вводные!B22*3+Вводные!B12</f>
+        <v>197.688</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="B17" s="15" t="n">
         <f aca="false">B12-B16</f>
-        <v>2184.312</v>
+        <v>2136.312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>